<commit_message>
Added filters to summary.xlsx
</commit_message>
<xml_diff>
--- a/analysis/summary.xlsx
+++ b/analysis/summary.xlsx
@@ -8,14 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\catalyst-tools\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6CB0D04-1D03-4898-ADE5-0C80CBCF1D9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CFCE0F1-A150-49F7-89FF-A7F3573A3B7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37640" yWindow="3030" windowWidth="36750" windowHeight="19860" xr2:uid="{DD260F35-B0C6-41E4-9255-0D5718BE7328}"/>
+    <workbookView xWindow="-37550" yWindow="3360" windowWidth="36750" windowHeight="18470" activeTab="1" xr2:uid="{DD260F35-B0C6-41E4-9255-0D5718BE7328}"/>
   </bookViews>
   <sheets>
     <sheet name="SegThy" sheetId="1" r:id="rId1"/>
     <sheet name="Synthetic" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SegThy!$A$1:$AC$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Synthetic!$A$1:$AC$17</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -4134,6 +4138,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AC33" xr:uid="{2DF80251-01B8-4EEE-BE3E-F00FCAF28141}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5626,6 +5631,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AC17" xr:uid="{64BC1F98-15C7-469E-BB0C-F6C580CA5A51}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Model F training, Model B analysis
- excel files containing Model B postprocessed data
- Model F training files, results, checkpoints
</commit_message>
<xml_diff>
--- a/analysis/summary.xlsx
+++ b/analysis/summary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\catalyst-tools\analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\catalyst-tools\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CFCE0F1-A150-49F7-89FF-A7F3573A3B7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A2CBD2-1AAA-46DC-9D7B-A805D7A0505F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37550" yWindow="3360" windowWidth="36750" windowHeight="18470" activeTab="1" xr2:uid="{DD260F35-B0C6-41E4-9255-0D5718BE7328}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DD260F35-B0C6-41E4-9255-0D5718BE7328}"/>
   </bookViews>
   <sheets>
     <sheet name="SegThy" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,20 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SegThy!$A$1:$AC$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Synthetic!$A$1:$AC$17</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1301,26 +1314,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DF80251-01B8-4EEE-BE3E-F00FCAF28141}">
   <dimension ref="A1:AC33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.27734375" customWidth="1"/>
-    <col min="2" max="2" width="23.27734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.28515625" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="5.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="12" width="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.27734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.0546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="23" max="28" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="3" customFormat="1" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:29" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1409,15 +1422,15 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D2" s="2">
         <v>0.11999999731779</v>
@@ -1429,164 +1442,164 @@
         <v>0.11999999731779</v>
       </c>
       <c r="G2">
-        <v>486</v>
+        <v>472</v>
       </c>
       <c r="H2">
-        <v>453</v>
+        <v>427</v>
       </c>
       <c r="I2">
-        <v>370</v>
+        <v>489</v>
       </c>
       <c r="J2" s="2">
-        <v>58.319998696446397</v>
+        <v>56.639998733997302</v>
       </c>
       <c r="K2" s="2">
-        <v>54.359998784959302</v>
+        <v>51.239998854696701</v>
       </c>
       <c r="L2" s="2">
-        <v>44.399999007582601</v>
+        <v>58.679998688399699</v>
       </c>
       <c r="M2">
-        <v>370</v>
+        <v>489</v>
       </c>
       <c r="N2">
-        <v>276</v>
+        <v>331</v>
       </c>
       <c r="O2">
-        <v>276</v>
+        <v>331</v>
       </c>
       <c r="P2" s="2">
-        <v>1.9295999137401501</v>
+        <v>1.43999993562698E-2</v>
       </c>
       <c r="Q2" s="2">
-        <v>74.001596691870702</v>
+        <v>142.775993617415</v>
       </c>
       <c r="R2" s="2">
-        <v>53.686745426102298</v>
+        <v>111.281324330472</v>
       </c>
       <c r="S2" s="2">
-        <v>13.823537777766999</v>
+        <v>32.011602186067798</v>
       </c>
       <c r="T2" s="2">
-        <v>-6.4689563966764299</v>
+        <v>-17.764085121910899</v>
       </c>
       <c r="U2" s="2">
-        <v>27.020508617068</v>
+        <v>7.5768040120629596</v>
       </c>
       <c r="V2" s="2">
-        <v>7.7505624307560996</v>
+        <v>-6.9057986387900696</v>
       </c>
       <c r="W2" s="2">
-        <v>11.0199623395274</v>
+        <v>7.4486649830511196</v>
       </c>
       <c r="X2" s="2">
-        <v>1.77810496876876</v>
+        <v>4.4200941036095802</v>
       </c>
       <c r="Y2" s="2">
-        <v>0.22110990141696499</v>
+        <v>0.13502681095887101</v>
       </c>
       <c r="Z2" s="2">
-        <v>0.67355746492965096</v>
+        <v>0.59387736681193704</v>
       </c>
       <c r="AA2" s="2">
-        <v>0.52575850864376605</v>
+        <v>0.52430916449558396</v>
       </c>
       <c r="AB2" s="2">
-        <v>7.3455279451867195E-2</v>
+        <v>5.9911369574359802E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="C3" t="s">
         <v>34</v>
       </c>
       <c r="D3" s="2">
-        <v>0.11999999731779</v>
+        <v>0.109999999403953</v>
       </c>
       <c r="E3" s="2">
-        <v>0.11999999731779</v>
+        <v>0.109999999403953</v>
       </c>
       <c r="F3" s="2">
-        <v>0.11999999731779</v>
+        <v>0.109999999403953</v>
       </c>
       <c r="G3">
-        <v>496</v>
+        <v>552</v>
       </c>
       <c r="H3">
-        <v>404</v>
+        <v>486</v>
       </c>
       <c r="I3">
-        <v>396</v>
+        <v>631</v>
       </c>
       <c r="J3" s="2">
-        <v>59.5199986696243</v>
+        <v>60.719999670982297</v>
       </c>
       <c r="K3" s="2">
-        <v>48.479998916387501</v>
+        <v>53.459999710321398</v>
       </c>
       <c r="L3" s="2">
-        <v>47.519998937845202</v>
+        <v>69.409999623894606</v>
       </c>
       <c r="M3">
-        <v>396</v>
+        <v>631</v>
       </c>
       <c r="N3">
-        <v>257</v>
+        <v>549</v>
       </c>
       <c r="O3">
-        <v>257</v>
+        <v>549</v>
       </c>
       <c r="P3" s="2">
-        <v>0.34559998455047602</v>
+        <v>2.8192999694466501</v>
       </c>
       <c r="Q3" s="2">
-        <v>16.3151992706537</v>
+        <v>120.721698691713</v>
       </c>
       <c r="R3" s="2">
-        <v>8.9000400690632606</v>
+        <v>93.169932870079407</v>
       </c>
       <c r="S3" s="2">
-        <v>3.2383094064033</v>
+        <v>16.0947907634228</v>
       </c>
       <c r="T3" s="2">
-        <v>-17.718737569616302</v>
+        <v>-18.237536257093801</v>
       </c>
       <c r="U3" s="2">
-        <v>1.1242703657935</v>
+        <v>14.1624125621047</v>
       </c>
       <c r="V3" s="2">
-        <v>-5.1390677634215702</v>
+        <v>-2.3463339584128802</v>
       </c>
       <c r="W3" s="2">
-        <v>5.4008666819821496</v>
+        <v>9.8254316126723698</v>
       </c>
       <c r="X3" s="2">
-        <v>0.27447722959486598</v>
+        <v>5.6265322155361401</v>
       </c>
       <c r="Y3" s="2">
-        <v>0.28683732101911702</v>
+        <v>0.12441874494572</v>
       </c>
       <c r="Z3" s="2">
-        <v>0.75398223686154997</v>
+        <v>0.62690660722956504</v>
       </c>
       <c r="AA3" s="2">
-        <v>0.45436411435693602</v>
+        <v>0.52255430541762404</v>
       </c>
       <c r="AB3" s="2">
-        <v>9.5494725170903294E-2</v>
+        <v>6.7018465924335996E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="C4" t="s">
         <v>31</v>
@@ -1601,78 +1614,78 @@
         <v>0.11999999731779</v>
       </c>
       <c r="G4">
-        <v>527</v>
+        <v>471</v>
       </c>
       <c r="H4">
-        <v>507</v>
+        <v>431</v>
       </c>
       <c r="I4">
-        <v>597</v>
+        <v>445</v>
       </c>
       <c r="J4" s="2">
-        <v>63.239998586475799</v>
+        <v>56.519998736679497</v>
       </c>
       <c r="K4" s="2">
-        <v>60.839998640120001</v>
+        <v>51.7199988439679</v>
       </c>
       <c r="L4" s="2">
-        <v>71.639998398721204</v>
+        <v>53.399998806416903</v>
       </c>
       <c r="M4">
-        <v>597</v>
+        <v>445</v>
       </c>
       <c r="N4">
-        <v>238</v>
+        <v>376</v>
       </c>
       <c r="O4">
-        <v>238</v>
+        <v>376</v>
       </c>
       <c r="P4" s="2">
-        <v>0.33119998519420601</v>
+        <v>2.8799998712539601E-2</v>
       </c>
       <c r="Q4" s="2">
-        <v>54.849597548031802</v>
+        <v>111.98879499371</v>
       </c>
       <c r="R4" s="2">
-        <v>28.597491158567198</v>
+        <v>87.996634364116105</v>
       </c>
       <c r="S4" s="2">
-        <v>15.556679666242401</v>
+        <v>19.765226094346701</v>
       </c>
       <c r="T4" s="2">
-        <v>-28.308785988929198</v>
+        <v>1.9560251279159999</v>
       </c>
       <c r="U4" s="2">
-        <v>-8.0751989851347901</v>
+        <v>62.470636235656798</v>
       </c>
       <c r="V4" s="2">
-        <v>-15.4238115480199</v>
+        <v>15.2511200646143</v>
       </c>
       <c r="W4" s="2">
-        <v>5.9903407238555397</v>
+        <v>6.5029202715596899</v>
       </c>
       <c r="X4" s="2">
-        <v>0.81674432923302198</v>
+        <v>3.9704080537633799</v>
       </c>
       <c r="Y4" s="2">
-        <v>0.387850944887628</v>
+        <v>9.9284713283697201E-2</v>
       </c>
       <c r="Z4" s="2">
-        <v>0.66283726481295702</v>
+        <v>0.64639713394496501</v>
       </c>
       <c r="AA4" s="2">
-        <v>0.54954347345696497</v>
+        <v>0.53986578454387801</v>
       </c>
       <c r="AB4" s="2">
-        <v>7.1455772085986802E-2</v>
+        <v>8.6976029628456103E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
         <v>34</v>
@@ -1687,81 +1700,81 @@
         <v>0.11999999731779</v>
       </c>
       <c r="G5">
-        <v>501</v>
+        <v>617</v>
       </c>
       <c r="H5">
-        <v>516</v>
+        <v>427</v>
       </c>
       <c r="I5">
-        <v>625</v>
+        <v>458</v>
       </c>
       <c r="J5" s="2">
-        <v>60.119998656213198</v>
+        <v>74.039998345076995</v>
       </c>
       <c r="K5" s="2">
-        <v>61.919998615980099</v>
+        <v>51.239998854696701</v>
       </c>
       <c r="L5" s="2">
-        <v>74.999998323619295</v>
+        <v>54.9599987715482</v>
       </c>
       <c r="M5">
-        <v>625</v>
+        <v>458</v>
       </c>
       <c r="N5">
-        <v>189</v>
+        <v>272</v>
       </c>
       <c r="O5">
-        <v>189</v>
+        <v>260</v>
       </c>
       <c r="P5" s="2">
-        <v>0.14399999356269799</v>
+        <v>5.7599997425079298E-2</v>
       </c>
       <c r="Q5" s="2">
-        <v>19.1663991431951</v>
+        <v>106.732795228672</v>
       </c>
       <c r="R5" s="2">
-        <v>10.301713825191699</v>
+        <v>73.351214368003895</v>
       </c>
       <c r="S5" s="2">
-        <v>5.88375254411425</v>
+        <v>20.132950239839399</v>
       </c>
       <c r="T5" s="2">
-        <v>5.6429962496727804</v>
+        <v>-25.688411047467099</v>
       </c>
       <c r="U5" s="2">
-        <v>9.4515843436410396</v>
+        <v>-3.74485725024959</v>
       </c>
       <c r="V5" s="2">
-        <v>7.4012167862119904</v>
+        <v>-11.593751892128401</v>
       </c>
       <c r="W5" s="2">
-        <v>0.92234835893643996</v>
+        <v>6.6536709204526598</v>
       </c>
       <c r="X5" s="2">
-        <v>0.233642864333024</v>
+        <v>2.3941835834574698</v>
       </c>
       <c r="Y5" s="2">
-        <v>0.17990560012635001</v>
+        <v>0.21955852797098899</v>
       </c>
       <c r="Z5" s="2">
-        <v>0.75630934253087601</v>
+        <v>0.59127803271340096</v>
       </c>
       <c r="AA5" s="2">
-        <v>0.48534067754822702</v>
+        <v>0.47887247583301201</v>
       </c>
       <c r="AB5" s="2">
-        <v>9.7658132006584297E-2</v>
+        <v>7.9653660189713205E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>93</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D6" s="2">
         <v>0.11999999731779</v>
@@ -1773,78 +1786,78 @@
         <v>0.11999999731779</v>
       </c>
       <c r="G6">
-        <v>493</v>
+        <v>512</v>
       </c>
       <c r="H6">
-        <v>444</v>
+        <v>430</v>
       </c>
       <c r="I6">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="J6" s="2">
-        <v>59.159998677670899</v>
+        <v>61.439998626708899</v>
       </c>
       <c r="K6" s="2">
-        <v>53.279998809099197</v>
+        <v>51.599998846650102</v>
       </c>
       <c r="L6" s="2">
-        <v>49.799998886883202</v>
+        <v>54.239998787641497</v>
       </c>
       <c r="M6">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="N6">
-        <v>276</v>
+        <v>398</v>
       </c>
       <c r="O6">
-        <v>276</v>
+        <v>398</v>
       </c>
       <c r="P6" s="2">
-        <v>0.84959996201992005</v>
+        <v>4.3199998068809503E-2</v>
       </c>
       <c r="Q6" s="2">
-        <v>17.279999227523799</v>
+        <v>83.807996253490401</v>
       </c>
       <c r="R6" s="2">
-        <v>10.401077795905101</v>
+        <v>67.971072338340505</v>
       </c>
       <c r="S6" s="2">
-        <v>2.71633372610582</v>
+        <v>11.2770149298498</v>
       </c>
       <c r="T6" s="2">
-        <v>22.781328024984099</v>
+        <v>-27.615261894174001</v>
       </c>
       <c r="U6" s="2">
-        <v>47.723491609628702</v>
+        <v>25.1242028815597</v>
       </c>
       <c r="V6" s="2">
-        <v>40.149546052521799</v>
+        <v>-15.5767199462778</v>
       </c>
       <c r="W6" s="2">
-        <v>7.5920641408914999</v>
+        <v>7.5223077608496096</v>
       </c>
       <c r="X6" s="2">
-        <v>0.34448368890056702</v>
+        <v>3.2462983423187199</v>
       </c>
       <c r="Y6" s="2">
-        <v>0.38660823879890699</v>
+        <v>9.7071870521207596E-2</v>
       </c>
       <c r="Z6" s="2">
-        <v>0.65624379874986705</v>
+        <v>0.67490278273135096</v>
       </c>
       <c r="AA6" s="2">
-        <v>0.50671206800679403</v>
+        <v>0.59877287891169595</v>
       </c>
       <c r="AB6" s="2">
-        <v>5.0269621417554498E-2</v>
+        <v>7.9645327854629494E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
         <v>34</v>
@@ -1859,422 +1872,422 @@
         <v>0.11999999731779</v>
       </c>
       <c r="G7">
-        <v>568</v>
+        <v>503</v>
       </c>
       <c r="H7">
-        <v>526</v>
+        <v>420</v>
       </c>
       <c r="I7">
-        <v>359</v>
+        <v>505</v>
       </c>
       <c r="J7" s="2">
-        <v>68.159998476505194</v>
+        <v>60.359998650848802</v>
       </c>
       <c r="K7" s="2">
-        <v>63.119998589158001</v>
+        <v>50.3999988734722</v>
       </c>
       <c r="L7" s="2">
-        <v>43.0799990370869</v>
+        <v>60.599998645484398</v>
       </c>
       <c r="M7">
-        <v>359</v>
+        <v>505</v>
       </c>
       <c r="N7">
-        <v>303</v>
+        <v>400</v>
       </c>
       <c r="O7">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="P7" s="2">
-        <v>0.17279999227523801</v>
+        <v>1.51199993240833</v>
       </c>
       <c r="Q7" s="2">
-        <v>29.505598680996901</v>
+        <v>94.031995796442004</v>
       </c>
       <c r="R7" s="2">
-        <v>19.5442209084834</v>
+        <v>67.600904978003896</v>
       </c>
       <c r="S7" s="2">
-        <v>4.8579998917373599</v>
+        <v>18.414478930946</v>
       </c>
       <c r="T7" s="2">
-        <v>-24.5180927952219</v>
+        <v>-20.3099124801046</v>
       </c>
       <c r="U7" s="2">
-        <v>8.6389556457861705</v>
+        <v>14.6549821547283</v>
       </c>
       <c r="V7" s="2">
-        <v>-8.3325068668936009</v>
+        <v>-9.8420890277294699</v>
       </c>
       <c r="W7" s="2">
-        <v>10.957687050472099</v>
+        <v>8.5874958321788792</v>
       </c>
       <c r="X7" s="2">
-        <v>0.71062785634868597</v>
+        <v>3.2448433664162799</v>
       </c>
       <c r="Y7" s="2">
-        <v>0.12855422849335099</v>
+        <v>0.25333749999203797</v>
       </c>
       <c r="Z7" s="2">
-        <v>0.62917649867069103</v>
+        <v>0.74799825085471205</v>
       </c>
       <c r="AA7" s="2">
-        <v>0.47129127136872401</v>
+        <v>0.59450010295019795</v>
       </c>
       <c r="AB7" s="2">
-        <v>7.8609768900081797E-2</v>
+        <v>6.1216842190851099E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C8" t="s">
         <v>31</v>
       </c>
       <c r="D8" s="2">
-        <v>0.11999999731779</v>
+        <v>0.109999999403953</v>
       </c>
       <c r="E8" s="2">
-        <v>0.11999999731779</v>
+        <v>0.109999999403953</v>
       </c>
       <c r="F8" s="2">
-        <v>0.11999999731779</v>
+        <v>0.109999999403953</v>
       </c>
       <c r="G8">
-        <v>462</v>
+        <v>480</v>
       </c>
       <c r="H8">
-        <v>408</v>
+        <v>389</v>
       </c>
       <c r="I8">
-        <v>431</v>
+        <v>395</v>
       </c>
       <c r="J8" s="2">
-        <v>55.4399987608194</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>127</v>
+        <v>52.799999713897698</v>
+      </c>
+      <c r="K8" s="2">
+        <v>42.789999768137903</v>
       </c>
       <c r="L8" s="2">
-        <v>51.7199988439679</v>
+        <v>43.449999764561603</v>
       </c>
       <c r="M8">
-        <v>431</v>
+        <v>395</v>
       </c>
       <c r="N8">
-        <v>318</v>
+        <v>342</v>
       </c>
       <c r="O8">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="P8" s="2">
-        <v>5.7599997425079298E-2</v>
+        <v>0.52029999436139995</v>
       </c>
       <c r="Q8" s="2">
-        <v>50.054397762393897</v>
+        <v>90.749999016523304</v>
       </c>
       <c r="R8" s="2">
-        <v>41.8799075617844</v>
+        <v>62.986655457751297</v>
       </c>
       <c r="S8" s="2">
-        <v>8.8783432890733902</v>
+        <v>21.106454943919299</v>
       </c>
       <c r="T8" s="2">
-        <v>-23.532565970836099</v>
+        <v>-25.664933140451701</v>
       </c>
       <c r="U8" s="2">
-        <v>24.876073134141301</v>
+        <v>1.9853568081245601</v>
       </c>
       <c r="V8" s="2">
-        <v>1.6638311699977399</v>
+        <v>-10.1384949178958</v>
       </c>
       <c r="W8" s="2">
-        <v>10.152222879209701</v>
+        <v>7.98598507078251</v>
       </c>
       <c r="X8" s="2">
-        <v>1.5981372368365401</v>
+        <v>2.3695579654809098</v>
       </c>
       <c r="Y8" s="2">
-        <v>0.35033518076395198</v>
+        <v>0.25493145248747001</v>
       </c>
       <c r="Z8" s="2">
-        <v>0.73347101209844301</v>
+        <v>0.86456629826791098</v>
       </c>
       <c r="AA8" s="2">
-        <v>0.59962098599737701</v>
+        <v>0.59640748296301105</v>
       </c>
       <c r="AB8" s="2">
-        <v>5.9412216987753098E-2</v>
+        <v>6.3317605429580398E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E9" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G9">
+        <v>486</v>
+      </c>
+      <c r="H9">
+        <v>453</v>
+      </c>
+      <c r="I9">
+        <v>370</v>
+      </c>
+      <c r="J9" s="2">
+        <v>58.319998696446397</v>
+      </c>
+      <c r="K9" s="2">
+        <v>54.359998784959302</v>
+      </c>
+      <c r="L9" s="2">
+        <v>44.399999007582601</v>
+      </c>
+      <c r="M9">
+        <v>370</v>
+      </c>
+      <c r="N9">
+        <v>276</v>
+      </c>
+      <c r="O9">
+        <v>276</v>
+      </c>
+      <c r="P9" s="2">
+        <v>1.9295999137401501</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>74.001596691870702</v>
+      </c>
+      <c r="R9" s="2">
+        <v>53.686745426102298</v>
+      </c>
+      <c r="S9" s="2">
+        <v>13.823537777766999</v>
+      </c>
+      <c r="T9" s="2">
+        <v>-6.4689563966764299</v>
+      </c>
+      <c r="U9" s="2">
+        <v>27.020508617068</v>
+      </c>
+      <c r="V9" s="2">
+        <v>7.7505624307560996</v>
+      </c>
+      <c r="W9" s="2">
+        <v>11.0199623395274</v>
+      </c>
+      <c r="X9" s="2">
+        <v>1.77810496876876</v>
+      </c>
+      <c r="Y9" s="2">
+        <v>0.22110990141696499</v>
+      </c>
+      <c r="Z9" s="2">
+        <v>0.67355746492965096</v>
+      </c>
+      <c r="AA9" s="2">
+        <v>0.52575850864376605</v>
+      </c>
+      <c r="AB9" s="2">
+        <v>7.3455279451867195E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="E9" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="F9" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="G9">
-        <v>503</v>
-      </c>
-      <c r="H9">
-        <v>420</v>
-      </c>
-      <c r="I9">
-        <v>505</v>
-      </c>
-      <c r="J9" s="2">
-        <v>60.359998650848802</v>
-      </c>
-      <c r="K9" s="2">
-        <v>50.3999988734722</v>
-      </c>
-      <c r="L9" s="2">
-        <v>60.599998645484398</v>
-      </c>
-      <c r="M9">
-        <v>505</v>
-      </c>
-      <c r="N9">
-        <v>400</v>
-      </c>
-      <c r="O9">
-        <v>400</v>
-      </c>
-      <c r="P9" s="2">
-        <v>1.51199993240833</v>
-      </c>
-      <c r="Q9" s="2">
-        <v>94.031995796442004</v>
-      </c>
-      <c r="R9" s="2">
-        <v>67.600904978003896</v>
-      </c>
-      <c r="S9" s="2">
-        <v>18.414478930946</v>
-      </c>
-      <c r="T9" s="2">
-        <v>-20.3099124801046</v>
-      </c>
-      <c r="U9" s="2">
-        <v>14.6549821547283</v>
-      </c>
-      <c r="V9" s="2">
-        <v>-9.8420890277294699</v>
-      </c>
-      <c r="W9" s="2">
-        <v>8.5874958321788792</v>
-      </c>
-      <c r="X9" s="2">
-        <v>3.2448433664162799</v>
-      </c>
-      <c r="Y9" s="2">
-        <v>0.25333749999203797</v>
-      </c>
-      <c r="Z9" s="2">
-        <v>0.74799825085471205</v>
-      </c>
-      <c r="AA9" s="2">
-        <v>0.59450010295019795</v>
-      </c>
-      <c r="AB9" s="2">
-        <v>6.1216842190851099E-2</v>
+      <c r="D10" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G10">
+        <v>555</v>
+      </c>
+      <c r="H10">
+        <v>423</v>
+      </c>
+      <c r="I10">
+        <v>375</v>
+      </c>
+      <c r="J10" s="2">
+        <v>66.599998511373997</v>
+      </c>
+      <c r="K10" s="2">
+        <v>50.759998865425501</v>
+      </c>
+      <c r="L10" s="2">
+        <v>44.999998994171598</v>
+      </c>
+      <c r="M10">
+        <v>375</v>
+      </c>
+      <c r="N10">
+        <v>140</v>
+      </c>
+      <c r="O10">
+        <v>134</v>
+      </c>
+      <c r="P10" s="2">
+        <v>2.8799998712539601E-2</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>73.7855967015266</v>
+      </c>
+      <c r="R10" s="2">
+        <v>48.253369271477602</v>
+      </c>
+      <c r="S10" s="2">
+        <v>18.270585734597699</v>
+      </c>
+      <c r="T10" s="2">
+        <v>-46.967911960960798</v>
+      </c>
+      <c r="U10" s="2">
+        <v>-19.884664449836599</v>
+      </c>
+      <c r="V10" s="2">
+        <v>-23.558293913636501</v>
+      </c>
+      <c r="W10" s="2">
+        <v>5.5106454963992704</v>
+      </c>
+      <c r="X10" s="2">
+        <v>0.81065658564123699</v>
+      </c>
+      <c r="Y10" s="2">
+        <v>0.12811466768490401</v>
+      </c>
+      <c r="Z10" s="2">
+        <v>0.61262924517089901</v>
+      </c>
+      <c r="AA10" s="2">
+        <v>0.49088387453915</v>
+      </c>
+      <c r="AB10" s="2">
+        <v>0.108496849520999</v>
       </c>
     </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.75">
-      <c r="A10" t="s">
-        <v>47</v>
-      </c>
-      <c r="B10" t="s">
-        <v>48</v>
-      </c>
-      <c r="C10" t="s">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C11" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="2">
-        <v>0.109999999403953</v>
-      </c>
-      <c r="E10" s="2">
-        <v>0.109999999403953</v>
-      </c>
-      <c r="F10" s="2">
-        <v>0.109999999403953</v>
-      </c>
-      <c r="G10">
-        <v>480</v>
-      </c>
-      <c r="H10">
-        <v>389</v>
-      </c>
-      <c r="I10">
-        <v>395</v>
-      </c>
-      <c r="J10" s="2">
-        <v>52.799999713897698</v>
-      </c>
-      <c r="K10" s="2">
-        <v>42.789999768137903</v>
-      </c>
-      <c r="L10" s="2">
-        <v>43.449999764561603</v>
-      </c>
-      <c r="M10">
-        <v>395</v>
-      </c>
-      <c r="N10">
-        <v>342</v>
-      </c>
-      <c r="O10">
-        <v>324</v>
-      </c>
-      <c r="P10" s="2">
-        <v>0.52029999436139995</v>
-      </c>
-      <c r="Q10" s="2">
-        <v>90.749999016523304</v>
-      </c>
-      <c r="R10" s="2">
-        <v>62.986655457751297</v>
-      </c>
-      <c r="S10" s="2">
-        <v>21.106454943919299</v>
-      </c>
-      <c r="T10" s="2">
-        <v>-25.664933140451701</v>
-      </c>
-      <c r="U10" s="2">
-        <v>1.9853568081245601</v>
-      </c>
-      <c r="V10" s="2">
-        <v>-10.1384949178958</v>
-      </c>
-      <c r="W10" s="2">
-        <v>7.98598507078251</v>
-      </c>
-      <c r="X10" s="2">
-        <v>2.3695579654809098</v>
-      </c>
-      <c r="Y10" s="2">
-        <v>0.25493145248747001</v>
-      </c>
-      <c r="Z10" s="2">
-        <v>0.86456629826791098</v>
-      </c>
-      <c r="AA10" s="2">
-        <v>0.59640748296301105</v>
-      </c>
-      <c r="AB10" s="2">
-        <v>6.3317605429580398E-2</v>
+      <c r="D11" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G11">
+        <v>536</v>
+      </c>
+      <c r="H11">
+        <v>521</v>
+      </c>
+      <c r="I11">
+        <v>584</v>
+      </c>
+      <c r="J11" s="2">
+        <v>64.319998562335897</v>
+      </c>
+      <c r="K11" s="2">
+        <v>62.519998602569103</v>
+      </c>
+      <c r="L11" s="2">
+        <v>70.079998433589907</v>
+      </c>
+      <c r="M11">
+        <v>584</v>
+      </c>
+      <c r="N11">
+        <v>393</v>
+      </c>
+      <c r="O11">
+        <v>381</v>
+      </c>
+      <c r="P11" s="2">
+        <v>0.115199994850158</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>60.868797278952599</v>
+      </c>
+      <c r="R11" s="2">
+        <v>46.3905322773265</v>
+      </c>
+      <c r="S11" s="2">
+        <v>13.435491339866999</v>
+      </c>
+      <c r="T11" s="2">
+        <v>-3.1914997723557601</v>
+      </c>
+      <c r="U11" s="2">
+        <v>45.938782762473998</v>
+      </c>
+      <c r="V11" s="2">
+        <v>19.107941579070602</v>
+      </c>
+      <c r="W11" s="2">
+        <v>12.049508977116099</v>
+      </c>
+      <c r="X11" s="2">
+        <v>2.18777745329808</v>
+      </c>
+      <c r="Y11" s="2">
+        <v>0.23619153925271799</v>
+      </c>
+      <c r="Z11" s="2">
+        <v>0.69380443818948101</v>
+      </c>
+      <c r="AA11" s="2">
+        <v>0.56888181700722096</v>
+      </c>
+      <c r="AB11" s="2">
+        <v>7.5158251711053697E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.75">
-      <c r="A11" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" t="s">
-        <v>50</v>
-      </c>
-      <c r="C11" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" s="2">
-        <v>0.109999999403953</v>
-      </c>
-      <c r="E11" s="2">
-        <v>0.109999999403953</v>
-      </c>
-      <c r="F11" s="2">
-        <v>0.109999999403953</v>
-      </c>
-      <c r="G11">
-        <v>552</v>
-      </c>
-      <c r="H11">
-        <v>486</v>
-      </c>
-      <c r="I11">
-        <v>631</v>
-      </c>
-      <c r="J11" s="2">
-        <v>60.719999670982297</v>
-      </c>
-      <c r="K11" s="2">
-        <v>53.459999710321398</v>
-      </c>
-      <c r="L11" s="2">
-        <v>69.409999623894606</v>
-      </c>
-      <c r="M11">
-        <v>631</v>
-      </c>
-      <c r="N11">
-        <v>549</v>
-      </c>
-      <c r="O11">
-        <v>549</v>
-      </c>
-      <c r="P11" s="2">
-        <v>2.8192999694466501</v>
-      </c>
-      <c r="Q11" s="2">
-        <v>120.721698691713</v>
-      </c>
-      <c r="R11" s="2">
-        <v>93.169932870079407</v>
-      </c>
-      <c r="S11" s="2">
-        <v>16.0947907634228</v>
-      </c>
-      <c r="T11" s="2">
-        <v>-18.237536257093801</v>
-      </c>
-      <c r="U11" s="2">
-        <v>14.1624125621047</v>
-      </c>
-      <c r="V11" s="2">
-        <v>-2.3463339584128802</v>
-      </c>
-      <c r="W11" s="2">
-        <v>9.8254316126723698</v>
-      </c>
-      <c r="X11" s="2">
-        <v>5.6265322155361401</v>
-      </c>
-      <c r="Y11" s="2">
-        <v>0.12441874494572</v>
-      </c>
-      <c r="Z11" s="2">
-        <v>0.62690660722956504</v>
-      </c>
-      <c r="AA11" s="2">
-        <v>0.52255430541762404</v>
-      </c>
-      <c r="AB11" s="2">
-        <v>6.7018465924335996E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
         <v>31</v>
@@ -2289,422 +2302,422 @@
         <v>0.11999999731779</v>
       </c>
       <c r="G12">
+        <v>462</v>
+      </c>
+      <c r="H12">
+        <v>408</v>
+      </c>
+      <c r="I12">
+        <v>431</v>
+      </c>
+      <c r="J12" s="2">
+        <v>55.4399987608194</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="L12" s="2">
+        <v>51.7199988439679</v>
+      </c>
+      <c r="M12">
+        <v>431</v>
+      </c>
+      <c r="N12">
+        <v>318</v>
+      </c>
+      <c r="O12">
+        <v>318</v>
+      </c>
+      <c r="P12" s="2">
+        <v>5.7599997425079298E-2</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>50.054397762393897</v>
+      </c>
+      <c r="R12" s="2">
+        <v>41.8799075617844</v>
+      </c>
+      <c r="S12" s="2">
+        <v>8.8783432890733902</v>
+      </c>
+      <c r="T12" s="2">
+        <v>-23.532565970836099</v>
+      </c>
+      <c r="U12" s="2">
+        <v>24.876073134141301</v>
+      </c>
+      <c r="V12" s="2">
+        <v>1.6638311699977399</v>
+      </c>
+      <c r="W12" s="2">
+        <v>10.152222879209701</v>
+      </c>
+      <c r="X12" s="2">
+        <v>1.5981372368365401</v>
+      </c>
+      <c r="Y12" s="2">
+        <v>0.35033518076395198</v>
+      </c>
+      <c r="Z12" s="2">
+        <v>0.73347101209844301</v>
+      </c>
+      <c r="AA12" s="2">
+        <v>0.59962098599737701</v>
+      </c>
+      <c r="AB12" s="2">
+        <v>5.9412216987753098E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E13" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G13">
+        <v>507</v>
+      </c>
+      <c r="H13">
+        <v>480</v>
+      </c>
+      <c r="I13">
+        <v>567</v>
+      </c>
+      <c r="J13" s="2">
+        <v>60.839998640120001</v>
+      </c>
+      <c r="K13" s="2">
+        <v>57.599998712539602</v>
+      </c>
+      <c r="L13" s="2">
+        <v>68.039998479187403</v>
+      </c>
+      <c r="M13">
+        <v>567</v>
+      </c>
+      <c r="N13">
+        <v>473</v>
+      </c>
+      <c r="O13">
+        <v>473</v>
+      </c>
+      <c r="P13" s="2">
+        <v>0.115199994850158</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>72.590396754956203</v>
+      </c>
+      <c r="R13" s="2">
+        <v>32.385294112518103</v>
+      </c>
+      <c r="S13" s="2">
+        <v>15.326562163500499</v>
+      </c>
+      <c r="T13" s="2">
+        <v>-1.59280688897673</v>
+      </c>
+      <c r="U13" s="2">
+        <v>38.702431399926198</v>
+      </c>
+      <c r="V13" s="2">
+        <v>12.2910171632528</v>
+      </c>
+      <c r="W13" s="2">
+        <v>11.8919504088847</v>
+      </c>
+      <c r="X13" s="2">
+        <v>1.8381892527398001</v>
+      </c>
+      <c r="Y13" s="2">
+        <v>0.11394954450048</v>
+      </c>
+      <c r="Z13" s="2">
+        <v>0.54872876285580996</v>
+      </c>
+      <c r="AA13" s="2">
+        <v>0.426328774527649</v>
+      </c>
+      <c r="AB13" s="2">
+        <v>6.4062039505979093E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>77</v>
+      </c>
+      <c r="B14" t="s">
+        <v>78</v>
+      </c>
+      <c r="C14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E14" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G14">
+        <v>533</v>
+      </c>
+      <c r="H14">
+        <v>464</v>
+      </c>
+      <c r="I14">
+        <v>440</v>
+      </c>
+      <c r="J14" s="2">
+        <v>63.959998570382503</v>
+      </c>
+      <c r="K14" s="2">
+        <v>55.679998755455003</v>
+      </c>
+      <c r="L14" s="2">
+        <v>52.799998819827998</v>
+      </c>
+      <c r="M14">
+        <v>440</v>
+      </c>
+      <c r="N14">
+        <v>364</v>
+      </c>
+      <c r="O14">
+        <v>337</v>
+      </c>
+      <c r="P14" s="2">
+        <v>1.7423999221086499</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>50.500797742438301</v>
+      </c>
+      <c r="R14" s="2">
+        <v>32.348016136348498</v>
+      </c>
+      <c r="S14" s="2">
+        <v>8.1421562230672802</v>
+      </c>
+      <c r="T14" s="2">
+        <v>-20.527470393122201</v>
+      </c>
+      <c r="U14" s="2">
+        <v>6.2944695376730397</v>
+      </c>
+      <c r="V14" s="2">
+        <v>-8.72487054063307</v>
+      </c>
+      <c r="W14" s="2">
+        <v>7.6323523358807002</v>
+      </c>
+      <c r="X14" s="2">
+        <v>1.4129613132535499</v>
+      </c>
+      <c r="Y14" s="2">
+        <v>0.13514368714610001</v>
+      </c>
+      <c r="Z14" s="2">
+        <v>0.71858735554700304</v>
+      </c>
+      <c r="AA14" s="2">
+        <v>0.35762653325822802</v>
+      </c>
+      <c r="AB14" s="2">
+        <v>8.5734654338940702E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G15">
         <v>524</v>
       </c>
-      <c r="H12">
+      <c r="H15">
         <v>431</v>
       </c>
-      <c r="I12">
+      <c r="I15">
         <v>555</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J15" s="2">
         <v>62.879998594522398</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K15" s="2">
         <v>51.7199988439679</v>
       </c>
-      <c r="L12" s="2">
+      <c r="L15" s="2">
         <v>66.599998511373997</v>
       </c>
-      <c r="M12">
+      <c r="M15">
         <v>555</v>
       </c>
-      <c r="N12">
+      <c r="N15">
         <v>436</v>
       </c>
-      <c r="O12">
+      <c r="O15">
         <v>436</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P15" s="2">
         <v>1.43999993562698E-2</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q15" s="2">
         <v>58.579197381305697</v>
       </c>
-      <c r="R12" s="2">
+      <c r="R15" s="2">
         <v>31.868453621240601</v>
       </c>
-      <c r="S12" s="2">
+      <c r="S15" s="2">
         <v>13.9120052690014</v>
       </c>
-      <c r="T12" s="2">
+      <c r="T15" s="2">
         <v>25.186266607769898</v>
       </c>
-      <c r="U12" s="2">
+      <c r="U15" s="2">
         <v>101.374821812148</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V15" s="2">
         <v>50.411150515860101</v>
       </c>
-      <c r="W12" s="2">
+      <c r="W15" s="2">
         <v>23.583712741471999</v>
       </c>
-      <c r="X12" s="2">
+      <c r="X15" s="2">
         <v>1.66735745619496</v>
       </c>
-      <c r="Y12" s="2">
+      <c r="Y15" s="2">
         <v>0.13424628943389499</v>
       </c>
-      <c r="Z12" s="2">
+      <c r="Z15" s="2">
         <v>0.81448698426402</v>
       </c>
-      <c r="AA12" s="2">
+      <c r="AA15" s="2">
         <v>0.502708268688002</v>
       </c>
-      <c r="AB12" s="2">
+      <c r="AB15" s="2">
         <v>8.0331869607131998E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.75">
-      <c r="A13" t="s">
-        <v>53</v>
-      </c>
-      <c r="B13" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" t="s">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>89</v>
+      </c>
+      <c r="B16" t="s">
+        <v>90</v>
+      </c>
+      <c r="C16" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="E13" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="F13" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="G13">
-        <v>617</v>
-      </c>
-      <c r="H13">
-        <v>427</v>
-      </c>
-      <c r="I13">
-        <v>458</v>
-      </c>
-      <c r="J13" s="2">
-        <v>74.039998345076995</v>
-      </c>
-      <c r="K13" s="2">
-        <v>51.239998854696701</v>
-      </c>
-      <c r="L13" s="2">
-        <v>54.9599987715482</v>
-      </c>
-      <c r="M13">
-        <v>458</v>
-      </c>
-      <c r="N13">
-        <v>272</v>
-      </c>
-      <c r="O13">
-        <v>260</v>
-      </c>
-      <c r="P13" s="2">
-        <v>5.7599997425079298E-2</v>
-      </c>
-      <c r="Q13" s="2">
-        <v>106.732795228672</v>
-      </c>
-      <c r="R13" s="2">
-        <v>73.351214368003895</v>
-      </c>
-      <c r="S13" s="2">
-        <v>20.132950239839399</v>
-      </c>
-      <c r="T13" s="2">
-        <v>-25.688411047467099</v>
-      </c>
-      <c r="U13" s="2">
-        <v>-3.74485725024959</v>
-      </c>
-      <c r="V13" s="2">
-        <v>-11.593751892128401</v>
-      </c>
-      <c r="W13" s="2">
-        <v>6.6536709204526598</v>
-      </c>
-      <c r="X13" s="2">
-        <v>2.3941835834574698</v>
-      </c>
-      <c r="Y13" s="2">
-        <v>0.21955852797098899</v>
-      </c>
-      <c r="Z13" s="2">
-        <v>0.59127803271340096</v>
-      </c>
-      <c r="AA13" s="2">
-        <v>0.47887247583301201</v>
-      </c>
-      <c r="AB13" s="2">
-        <v>7.9653660189713205E-2</v>
+      <c r="D16" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E16" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G16">
+        <v>588</v>
+      </c>
+      <c r="H16">
+        <v>514</v>
+      </c>
+      <c r="I16">
+        <v>696</v>
+      </c>
+      <c r="J16" s="2">
+        <v>70.559998422861099</v>
+      </c>
+      <c r="K16" s="2">
+        <v>61.679998621344502</v>
+      </c>
+      <c r="L16" s="2">
+        <v>83.519998133182497</v>
+      </c>
+      <c r="M16">
+        <v>696</v>
+      </c>
+      <c r="N16">
+        <v>530</v>
+      </c>
+      <c r="O16">
+        <v>530</v>
+      </c>
+      <c r="P16" s="2">
+        <v>0.54719997553825395</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>40.535998187899601</v>
+      </c>
+      <c r="R16" s="2">
+        <v>28.883790406907099</v>
+      </c>
+      <c r="S16" s="2">
+        <v>7.8649864410657599</v>
+      </c>
+      <c r="T16" s="2">
+        <v>-24.743954745608399</v>
+      </c>
+      <c r="U16" s="2">
+        <v>9.7046363882575104</v>
+      </c>
+      <c r="V16" s="2">
+        <v>0.83436034278634796</v>
+      </c>
+      <c r="W16" s="2">
+        <v>8.0313582978660207</v>
+      </c>
+      <c r="X16" s="2">
+        <v>1.83700902881894</v>
+      </c>
+      <c r="Y16" s="2">
+        <v>0.11867453863633599</v>
+      </c>
+      <c r="Z16" s="2">
+        <v>0.70639361441663895</v>
+      </c>
+      <c r="AA16" s="2">
+        <v>0.39402604452571399</v>
+      </c>
+      <c r="AB16" s="2">
+        <v>0.145607079988959</v>
       </c>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.75">
-      <c r="A14" t="s">
-        <v>55</v>
-      </c>
-      <c r="B14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C14" t="s">
-        <v>31</v>
-      </c>
-      <c r="D14" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="E14" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="F14" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="G14">
-        <v>471</v>
-      </c>
-      <c r="H14">
-        <v>431</v>
-      </c>
-      <c r="I14">
-        <v>445</v>
-      </c>
-      <c r="J14" s="2">
-        <v>56.519998736679497</v>
-      </c>
-      <c r="K14" s="2">
-        <v>51.7199988439679</v>
-      </c>
-      <c r="L14" s="2">
-        <v>53.399998806416903</v>
-      </c>
-      <c r="M14">
-        <v>445</v>
-      </c>
-      <c r="N14">
-        <v>376</v>
-      </c>
-      <c r="O14">
-        <v>376</v>
-      </c>
-      <c r="P14" s="2">
-        <v>2.8799998712539601E-2</v>
-      </c>
-      <c r="Q14" s="2">
-        <v>111.98879499371</v>
-      </c>
-      <c r="R14" s="2">
-        <v>87.996634364116105</v>
-      </c>
-      <c r="S14" s="2">
-        <v>19.765226094346701</v>
-      </c>
-      <c r="T14" s="2">
-        <v>1.9560251279159999</v>
-      </c>
-      <c r="U14" s="2">
-        <v>62.470636235656798</v>
-      </c>
-      <c r="V14" s="2">
-        <v>15.2511200646143</v>
-      </c>
-      <c r="W14" s="2">
-        <v>6.5029202715596899</v>
-      </c>
-      <c r="X14" s="2">
-        <v>3.9704080537633799</v>
-      </c>
-      <c r="Y14" s="2">
-        <v>9.9284713283697201E-2</v>
-      </c>
-      <c r="Z14" s="2">
-        <v>0.64639713394496501</v>
-      </c>
-      <c r="AA14" s="2">
-        <v>0.53986578454387801</v>
-      </c>
-      <c r="AB14" s="2">
-        <v>8.6976029628456103E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.75">
-      <c r="A15" t="s">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>57</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B17" t="s">
         <v>58</v>
-      </c>
-      <c r="C15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="E15" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="F15" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="G15">
-        <v>531</v>
-      </c>
-      <c r="H15">
-        <v>425</v>
-      </c>
-      <c r="I15">
-        <v>454</v>
-      </c>
-      <c r="J15" s="2">
-        <v>63.719998575746999</v>
-      </c>
-      <c r="K15" s="2">
-        <v>50.999998860061098</v>
-      </c>
-      <c r="L15" s="2">
-        <v>54.4799987822771</v>
-      </c>
-      <c r="M15">
-        <v>454</v>
-      </c>
-      <c r="N15">
-        <v>378</v>
-      </c>
-      <c r="O15">
-        <v>378</v>
-      </c>
-      <c r="P15" s="2">
-        <v>0.187199991631507</v>
-      </c>
-      <c r="Q15" s="2">
-        <v>39.758398222661</v>
-      </c>
-      <c r="R15" s="2">
-        <v>28.850893948359701</v>
-      </c>
-      <c r="S15" s="2">
-        <v>7.4287949192359397</v>
-      </c>
-      <c r="T15" s="2">
-        <v>-30.9667451724359</v>
-      </c>
-      <c r="U15" s="2">
-        <v>0.44713152855322502</v>
-      </c>
-      <c r="V15" s="2">
-        <v>-12.4930100104218</v>
-      </c>
-      <c r="W15" s="2">
-        <v>9.9024235422562494</v>
-      </c>
-      <c r="X15" s="2">
-        <v>1.3086765202463899</v>
-      </c>
-      <c r="Y15" s="2">
-        <v>8.4750056949813607E-2</v>
-      </c>
-      <c r="Z15" s="2">
-        <v>0.70522260449927798</v>
-      </c>
-      <c r="AA15" s="2">
-        <v>0.59660376373724699</v>
-      </c>
-      <c r="AB15" s="2">
-        <v>7.6115359300433005E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.75">
-      <c r="A16" t="s">
-        <v>59</v>
-      </c>
-      <c r="B16" t="s">
-        <v>60</v>
-      </c>
-      <c r="C16" t="s">
-        <v>31</v>
-      </c>
-      <c r="D16" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="E16" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="F16" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="G16">
-        <v>487</v>
-      </c>
-      <c r="H16">
-        <v>399</v>
-      </c>
-      <c r="I16">
-        <v>530</v>
-      </c>
-      <c r="J16" s="2">
-        <v>58.439998693764203</v>
-      </c>
-      <c r="K16" s="2">
-        <v>47.879998929798603</v>
-      </c>
-      <c r="L16" s="2">
-        <v>63.599998578429201</v>
-      </c>
-      <c r="M16">
-        <v>530</v>
-      </c>
-      <c r="N16">
-        <v>339</v>
-      </c>
-      <c r="O16">
-        <v>339</v>
-      </c>
-      <c r="P16" s="2">
-        <v>0.53279997618198405</v>
-      </c>
-      <c r="Q16" s="2">
-        <v>56.131197490739801</v>
-      </c>
-      <c r="R16" s="2">
-        <v>26.435255455419998</v>
-      </c>
-      <c r="S16" s="2">
-        <v>12.7292637322999</v>
-      </c>
-      <c r="T16" s="2">
-        <v>-8.2186476495978606</v>
-      </c>
-      <c r="U16" s="2">
-        <v>36.7989606053698</v>
-      </c>
-      <c r="V16" s="2">
-        <v>21.8704590079608</v>
-      </c>
-      <c r="W16" s="2">
-        <v>7.6048811334331701</v>
-      </c>
-      <c r="X16" s="2">
-        <v>1.0753861678897301</v>
-      </c>
-      <c r="Y16" s="2">
-        <v>0.220336162301324</v>
-      </c>
-      <c r="Z16" s="2">
-        <v>0.72019274276490997</v>
-      </c>
-      <c r="AA16" s="2">
-        <v>0.52910233574810595</v>
-      </c>
-      <c r="AB16" s="2">
-        <v>0.13861466829032101</v>
-      </c>
-    </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.75">
-      <c r="A17" t="s">
-        <v>61</v>
-      </c>
-      <c r="B17" t="s">
-        <v>62</v>
       </c>
       <c r="C17" t="s">
         <v>34</v>
@@ -2719,78 +2732,78 @@
         <v>0.11999999731779</v>
       </c>
       <c r="G17">
-        <v>472</v>
+        <v>531</v>
       </c>
       <c r="H17">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="I17">
-        <v>489</v>
+        <v>454</v>
       </c>
       <c r="J17" s="2">
-        <v>56.639998733997302</v>
+        <v>63.719998575746999</v>
       </c>
       <c r="K17" s="2">
-        <v>51.239998854696701</v>
+        <v>50.999998860061098</v>
       </c>
       <c r="L17" s="2">
-        <v>58.679998688399699</v>
+        <v>54.4799987822771</v>
       </c>
       <c r="M17">
-        <v>489</v>
+        <v>454</v>
       </c>
       <c r="N17">
-        <v>331</v>
+        <v>378</v>
       </c>
       <c r="O17">
-        <v>331</v>
+        <v>378</v>
       </c>
       <c r="P17" s="2">
-        <v>1.43999993562698E-2</v>
+        <v>0.187199991631507</v>
       </c>
       <c r="Q17" s="2">
-        <v>142.775993617415</v>
+        <v>39.758398222661</v>
       </c>
       <c r="R17" s="2">
-        <v>111.281324330472</v>
+        <v>28.850893948359701</v>
       </c>
       <c r="S17" s="2">
-        <v>32.011602186067798</v>
+        <v>7.4287949192359397</v>
       </c>
       <c r="T17" s="2">
-        <v>-17.764085121910899</v>
+        <v>-30.9667451724359</v>
       </c>
       <c r="U17" s="2">
-        <v>7.5768040120629596</v>
+        <v>0.44713152855322502</v>
       </c>
       <c r="V17" s="2">
-        <v>-6.9057986387900696</v>
+        <v>-12.4930100104218</v>
       </c>
       <c r="W17" s="2">
-        <v>7.4486649830511196</v>
+        <v>9.9024235422562494</v>
       </c>
       <c r="X17" s="2">
-        <v>4.4200941036095802</v>
+        <v>1.3086765202463899</v>
       </c>
       <c r="Y17" s="2">
-        <v>0.13502681095887101</v>
+        <v>8.4750056949813607E-2</v>
       </c>
       <c r="Z17" s="2">
-        <v>0.59387736681193704</v>
+        <v>0.70522260449927798</v>
       </c>
       <c r="AA17" s="2">
-        <v>0.52430916449558396</v>
+        <v>0.59660376373724699</v>
       </c>
       <c r="AB17" s="2">
-        <v>5.9911369574359802E-2</v>
+        <v>7.6115359300433005E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.75">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="C18" t="s">
         <v>31</v>
@@ -2805,508 +2818,508 @@
         <v>0.11999999731779</v>
       </c>
       <c r="G18">
-        <v>500</v>
+        <v>527</v>
       </c>
       <c r="H18">
-        <v>442</v>
+        <v>507</v>
       </c>
       <c r="I18">
-        <v>479</v>
+        <v>597</v>
       </c>
       <c r="J18" s="2">
-        <v>59.9999986588954</v>
+        <v>63.239998586475799</v>
       </c>
       <c r="K18" s="2">
-        <v>53.039998814463601</v>
+        <v>60.839998640120001</v>
       </c>
       <c r="L18" s="2">
-        <v>57.479998715221797</v>
+        <v>71.639998398721204</v>
       </c>
       <c r="M18">
-        <v>479</v>
+        <v>597</v>
       </c>
       <c r="N18">
-        <v>281</v>
+        <v>238</v>
       </c>
       <c r="O18">
-        <v>281</v>
+        <v>238</v>
       </c>
       <c r="P18" s="2">
-        <v>0.100799995493888</v>
+        <v>0.33119998519420601</v>
       </c>
       <c r="Q18" s="2">
-        <v>10.0655995500326</v>
+        <v>54.849597548031802</v>
       </c>
       <c r="R18" s="2">
-        <v>6.2332523903910397</v>
+        <v>28.597491158567198</v>
       </c>
       <c r="S18" s="2">
-        <v>1.6164454200715701</v>
+        <v>15.556679666242401</v>
       </c>
       <c r="T18" s="2">
-        <v>5.5762378785484499</v>
+        <v>-28.308785988929198</v>
       </c>
       <c r="U18" s="2">
-        <v>52.288517561874002</v>
+        <v>-8.0751989851347901</v>
       </c>
       <c r="V18" s="2">
-        <v>28.889137936259299</v>
+        <v>-15.4238115480199</v>
       </c>
       <c r="W18" s="2">
-        <v>15.527761680313899</v>
+        <v>5.9903407238555397</v>
       </c>
       <c r="X18" s="2">
-        <v>0.210185265905978</v>
+        <v>0.81674432923302198</v>
       </c>
       <c r="Y18" s="2">
-        <v>0.50060688730810599</v>
+        <v>0.387850944887628</v>
       </c>
       <c r="Z18" s="2">
-        <v>0.87266462599716399</v>
+        <v>0.66283726481295702</v>
       </c>
       <c r="AA18" s="2">
-        <v>0.63383746204019498</v>
+        <v>0.54954347345696497</v>
       </c>
       <c r="AB18" s="2">
-        <v>5.19615440898075E-2</v>
+        <v>7.1455772085986802E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.75">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B19" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C19" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E19" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F19" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G19">
+        <v>487</v>
+      </c>
+      <c r="H19">
+        <v>399</v>
+      </c>
+      <c r="I19">
+        <v>530</v>
+      </c>
+      <c r="J19" s="2">
+        <v>58.439998693764203</v>
+      </c>
+      <c r="K19" s="2">
+        <v>47.879998929798603</v>
+      </c>
+      <c r="L19" s="2">
+        <v>63.599998578429201</v>
+      </c>
+      <c r="M19">
+        <v>530</v>
+      </c>
+      <c r="N19">
+        <v>339</v>
+      </c>
+      <c r="O19">
+        <v>339</v>
+      </c>
+      <c r="P19" s="2">
+        <v>0.53279997618198405</v>
+      </c>
+      <c r="Q19" s="2">
+        <v>56.131197490739801</v>
+      </c>
+      <c r="R19" s="2">
+        <v>26.435255455419998</v>
+      </c>
+      <c r="S19" s="2">
+        <v>12.7292637322999</v>
+      </c>
+      <c r="T19" s="2">
+        <v>-8.2186476495978606</v>
+      </c>
+      <c r="U19" s="2">
+        <v>36.7989606053698</v>
+      </c>
+      <c r="V19" s="2">
+        <v>21.8704590079608</v>
+      </c>
+      <c r="W19" s="2">
+        <v>7.6048811334331701</v>
+      </c>
+      <c r="X19" s="2">
+        <v>1.0753861678897301</v>
+      </c>
+      <c r="Y19" s="2">
+        <v>0.220336162301324</v>
+      </c>
+      <c r="Z19" s="2">
+        <v>0.72019274276490997</v>
+      </c>
+      <c r="AA19" s="2">
+        <v>0.52910233574810595</v>
+      </c>
+      <c r="AB19" s="2">
+        <v>0.13861466829032101</v>
+      </c>
+    </row>
+    <row r="20" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="E19" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="F19" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="G19">
-        <v>555</v>
-      </c>
-      <c r="H19">
-        <v>423</v>
-      </c>
-      <c r="I19">
-        <v>375</v>
-      </c>
-      <c r="J19" s="2">
-        <v>66.599998511373997</v>
-      </c>
-      <c r="K19" s="2">
-        <v>50.759998865425501</v>
-      </c>
-      <c r="L19" s="2">
-        <v>44.999998994171598</v>
-      </c>
-      <c r="M19">
-        <v>375</v>
-      </c>
-      <c r="N19">
-        <v>140</v>
-      </c>
-      <c r="O19">
-        <v>134</v>
-      </c>
-      <c r="P19" s="2">
-        <v>2.8799998712539601E-2</v>
-      </c>
-      <c r="Q19" s="2">
-        <v>73.7855967015266</v>
-      </c>
-      <c r="R19" s="2">
-        <v>48.253369271477602</v>
-      </c>
-      <c r="S19" s="2">
-        <v>18.270585734597699</v>
-      </c>
-      <c r="T19" s="2">
-        <v>-46.967911960960798</v>
-      </c>
-      <c r="U19" s="2">
-        <v>-19.884664449836599</v>
-      </c>
-      <c r="V19" s="2">
-        <v>-23.558293913636501</v>
-      </c>
-      <c r="W19" s="2">
-        <v>5.5106454963992704</v>
-      </c>
-      <c r="X19" s="2">
-        <v>0.81065658564123699</v>
-      </c>
-      <c r="Y19" s="2">
-        <v>0.12811466768490401</v>
-      </c>
-      <c r="Z19" s="2">
-        <v>0.61262924517089901</v>
-      </c>
-      <c r="AA19" s="2">
-        <v>0.49088387453915</v>
-      </c>
-      <c r="AB19" s="2">
-        <v>0.108496849520999</v>
+      <c r="D20" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E20" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F20" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G20">
+        <v>568</v>
+      </c>
+      <c r="H20">
+        <v>526</v>
+      </c>
+      <c r="I20">
+        <v>359</v>
+      </c>
+      <c r="J20" s="2">
+        <v>68.159998476505194</v>
+      </c>
+      <c r="K20" s="2">
+        <v>63.119998589158001</v>
+      </c>
+      <c r="L20" s="2">
+        <v>43.0799990370869</v>
+      </c>
+      <c r="M20">
+        <v>359</v>
+      </c>
+      <c r="N20">
+        <v>303</v>
+      </c>
+      <c r="O20">
+        <v>300</v>
+      </c>
+      <c r="P20" s="2">
+        <v>0.17279999227523801</v>
+      </c>
+      <c r="Q20" s="2">
+        <v>29.505598680996901</v>
+      </c>
+      <c r="R20" s="2">
+        <v>19.5442209084834</v>
+      </c>
+      <c r="S20" s="2">
+        <v>4.8579998917373599</v>
+      </c>
+      <c r="T20" s="2">
+        <v>-24.5180927952219</v>
+      </c>
+      <c r="U20" s="2">
+        <v>8.6389556457861705</v>
+      </c>
+      <c r="V20" s="2">
+        <v>-8.3325068668936009</v>
+      </c>
+      <c r="W20" s="2">
+        <v>10.957687050472099</v>
+      </c>
+      <c r="X20" s="2">
+        <v>0.71062785634868597</v>
+      </c>
+      <c r="Y20" s="2">
+        <v>0.12855422849335099</v>
+      </c>
+      <c r="Z20" s="2">
+        <v>0.62917649867069103</v>
+      </c>
+      <c r="AA20" s="2">
+        <v>0.47129127136872401</v>
+      </c>
+      <c r="AB20" s="2">
+        <v>7.8609768900081797E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.75">
-      <c r="A20" t="s">
-        <v>67</v>
-      </c>
-      <c r="B20" t="s">
-        <v>68</v>
-      </c>
-      <c r="C20" t="s">
-        <v>31</v>
-      </c>
-      <c r="D20" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="E20" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="F20" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="G20">
-        <v>492</v>
-      </c>
-      <c r="H20">
-        <v>493</v>
-      </c>
-      <c r="I20">
-        <v>470</v>
-      </c>
-      <c r="J20" s="2">
-        <v>59.039998680353101</v>
-      </c>
-      <c r="K20" s="2">
-        <v>59.159998677670899</v>
-      </c>
-      <c r="L20" s="2">
-        <v>56.399998739361699</v>
-      </c>
-      <c r="M20">
-        <v>470</v>
-      </c>
-      <c r="N20">
-        <v>409</v>
-      </c>
-      <c r="O20">
-        <v>408</v>
-      </c>
-      <c r="P20" s="2">
-        <v>0.100799995493888</v>
-      </c>
-      <c r="Q20" s="2">
-        <v>27.705598761463101</v>
-      </c>
-      <c r="R20" s="2">
-        <v>13.406540231976701</v>
-      </c>
-      <c r="S20" s="2">
-        <v>7.2227892634755397</v>
-      </c>
-      <c r="T20" s="2">
-        <v>-3.6791164126064002</v>
-      </c>
-      <c r="U20" s="2">
-        <v>48.885386689612801</v>
-      </c>
-      <c r="V20" s="2">
-        <v>11.991644925359401</v>
-      </c>
-      <c r="W20" s="2">
-        <v>11.7091698601528</v>
-      </c>
-      <c r="X20" s="2">
-        <v>0.65799297987812999</v>
-      </c>
-      <c r="Y20" s="2">
-        <v>0.245436926061702</v>
-      </c>
-      <c r="Z20" s="2">
-        <v>0.62831853071795796</v>
-      </c>
-      <c r="AA20" s="2">
-        <v>0.45913242350329603</v>
-      </c>
-      <c r="AB20" s="2">
-        <v>8.0821992081826305E-2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.75">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="C21" t="s">
         <v>34</v>
       </c>
       <c r="D21" s="2">
-        <v>0.11999999731779</v>
+        <v>0.109999999403953</v>
       </c>
       <c r="E21" s="2">
-        <v>0.11999999731779</v>
+        <v>0.109999999403953</v>
       </c>
       <c r="F21" s="2">
-        <v>0.11999999731779</v>
+        <v>0.109999999403953</v>
       </c>
       <c r="G21">
-        <v>509</v>
+        <v>604</v>
       </c>
       <c r="H21">
-        <v>419</v>
+        <v>482</v>
       </c>
       <c r="I21">
-        <v>470</v>
+        <v>546</v>
       </c>
       <c r="J21" s="2">
-        <v>61.079998634755597</v>
+        <v>66.439999639987903</v>
       </c>
       <c r="K21" s="2">
-        <v>50.279998876154401</v>
+        <v>53.019999712705598</v>
       </c>
       <c r="L21" s="2">
-        <v>56.399998739361699</v>
+        <v>60.059999674558597</v>
       </c>
       <c r="M21">
-        <v>470</v>
+        <v>546</v>
       </c>
       <c r="N21">
-        <v>421</v>
+        <v>376</v>
       </c>
       <c r="O21">
-        <v>421</v>
+        <v>376</v>
       </c>
       <c r="P21" s="2">
-        <v>0.17279999227523801</v>
+        <v>0.108899998819828</v>
       </c>
       <c r="Q21" s="2">
-        <v>19.238399139976501</v>
+        <v>41.865999546289402</v>
       </c>
       <c r="R21" s="2">
-        <v>9.4470494589191194</v>
+        <v>18.786537030448901</v>
       </c>
       <c r="S21" s="2">
-        <v>4.4674063575587502</v>
+        <v>9.9718519030673392</v>
       </c>
       <c r="T21" s="2">
-        <v>-37.377476810110601</v>
+        <v>-18.664611344916999</v>
       </c>
       <c r="U21" s="2">
-        <v>8.8260465440543907</v>
+        <v>8.4478220753991895</v>
       </c>
       <c r="V21" s="2">
-        <v>-9.3330666501601804</v>
+        <v>-8.6137667186061506</v>
       </c>
       <c r="W21" s="2">
-        <v>14.532382732052</v>
+        <v>8.9614095681574799</v>
       </c>
       <c r="X21" s="2">
-        <v>0.47726492799689102</v>
+        <v>0.77701116736905196</v>
       </c>
       <c r="Y21" s="2">
-        <v>0.17896940301683301</v>
+        <v>0.28972257847031402</v>
       </c>
       <c r="Z21" s="2">
-        <v>0.95660952773668395</v>
+        <v>1</v>
       </c>
       <c r="AA21" s="2">
-        <v>0.37852913096401303</v>
+        <v>0.53287827651128705</v>
       </c>
       <c r="AB21" s="2">
-        <v>9.7776851486295405E-2</v>
+        <v>8.59954147501025E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.75">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" t="s">
+        <v>82</v>
+      </c>
+      <c r="C22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E22" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F22" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G22">
+        <v>488</v>
+      </c>
+      <c r="H22">
+        <v>503</v>
+      </c>
+      <c r="I22">
+        <v>544</v>
+      </c>
+      <c r="J22" s="2">
+        <v>58.559998691082001</v>
+      </c>
+      <c r="K22" s="2">
+        <v>60.359998650848802</v>
+      </c>
+      <c r="L22" s="2">
+        <v>65.279998540878296</v>
+      </c>
+      <c r="M22">
+        <v>544</v>
+      </c>
+      <c r="N22">
+        <v>413</v>
+      </c>
+      <c r="O22">
+        <v>413</v>
+      </c>
+      <c r="P22" s="2">
+        <v>4.3199998068809503E-2</v>
+      </c>
+      <c r="Q22" s="2">
+        <v>33.883198485302898</v>
+      </c>
+      <c r="R22" s="2">
+        <v>16.1630404396833</v>
+      </c>
+      <c r="S22" s="2">
+        <v>5.5449052384811104</v>
+      </c>
+      <c r="T22" s="2">
+        <v>-30.113181857117699</v>
+      </c>
+      <c r="U22" s="2">
+        <v>14.5372308886172</v>
+      </c>
+      <c r="V22" s="2">
+        <v>-2.2214572979969098</v>
+      </c>
+      <c r="W22" s="2">
+        <v>10.317174022222501</v>
+      </c>
+      <c r="X22" s="2">
+        <v>0.80104026628606195</v>
+      </c>
+      <c r="Y22" s="2">
+        <v>0.21681631811889299</v>
+      </c>
+      <c r="Z22" s="2">
+        <v>0.73100770886853905</v>
+      </c>
+      <c r="AA22" s="2">
+        <v>0.40499463756417198</v>
+      </c>
+      <c r="AB22" s="2">
+        <v>0.12384299345529901</v>
+      </c>
+    </row>
+    <row r="23" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>71</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B23" t="s">
         <v>72</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C23" t="s">
         <v>31</v>
       </c>
-      <c r="D22" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="E22" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="F22" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="G22">
+      <c r="D23" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E23" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F23" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G23">
         <v>590</v>
       </c>
-      <c r="H22">
+      <c r="H23">
         <v>482</v>
       </c>
-      <c r="I22">
+      <c r="I23">
         <v>563</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J23" s="2">
         <v>70.799998417496596</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K23" s="2">
         <v>57.839998707175198</v>
       </c>
-      <c r="L22" s="2">
+      <c r="L23" s="2">
         <v>67.559998489916296</v>
       </c>
-      <c r="M22">
+      <c r="M23">
         <v>563</v>
       </c>
-      <c r="N22">
+      <c r="N23">
         <v>214</v>
       </c>
-      <c r="O22">
+      <c r="O23">
         <v>214</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P23" s="2">
         <v>0.14399999356269799</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q23" s="2">
         <v>27.2303987827062</v>
       </c>
-      <c r="R22" s="2">
+      <c r="R23" s="2">
         <v>15.352014266982399</v>
       </c>
-      <c r="S22" s="2">
+      <c r="S23" s="2">
         <v>8.5225484868254799</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T23" s="2">
         <v>-5.97240811185649</v>
       </c>
-      <c r="U22" s="2">
+      <c r="U23" s="2">
         <v>2.9837405345386898</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V23" s="2">
         <v>-2.07456074831292</v>
       </c>
-      <c r="W22" s="2">
+      <c r="W23" s="2">
         <v>2.0110854069563699</v>
       </c>
-      <c r="X22" s="2">
+      <c r="X23" s="2">
         <v>0.39423971756416498</v>
       </c>
-      <c r="Y22" s="2">
+      <c r="Y23" s="2">
         <v>0.19277623004758901</v>
       </c>
-      <c r="Z22" s="2">
+      <c r="Z23" s="2">
         <v>0.65037135243857702</v>
       </c>
-      <c r="AA22" s="2">
+      <c r="AA23" s="2">
         <v>0.44869324601136701</v>
       </c>
-      <c r="AB22" s="2">
+      <c r="AB23" s="2">
         <v>0.103399049684227</v>
       </c>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.75">
-      <c r="A23" t="s">
-        <v>73</v>
-      </c>
-      <c r="B23" t="s">
-        <v>74</v>
-      </c>
-      <c r="C23" t="s">
-        <v>34</v>
-      </c>
-      <c r="D23" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="E23" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="F23" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="G23">
-        <v>457</v>
-      </c>
-      <c r="H23">
-        <v>503</v>
-      </c>
-      <c r="I23">
-        <v>530</v>
-      </c>
-      <c r="J23" s="2">
-        <v>54.839998774230402</v>
-      </c>
-      <c r="K23" s="2">
-        <v>60.359998650848802</v>
-      </c>
-      <c r="L23" s="2">
-        <v>63.599998578429201</v>
-      </c>
-      <c r="M23">
-        <v>530</v>
-      </c>
-      <c r="N23">
-        <v>348</v>
-      </c>
-      <c r="O23">
-        <v>348</v>
-      </c>
-      <c r="P23" s="2">
-        <v>0.41759998133182502</v>
-      </c>
-      <c r="Q23" s="2">
-        <v>19.915199109721101</v>
-      </c>
-      <c r="R23" s="2">
-        <v>11.121599502825701</v>
-      </c>
-      <c r="S23" s="2">
-        <v>5.7592023770084904</v>
-      </c>
-      <c r="T23" s="2">
-        <v>-19.800098712087902</v>
-      </c>
-      <c r="U23" s="2">
-        <v>1.55906942884642</v>
-      </c>
-      <c r="V23" s="2">
-        <v>-6.89808119767501</v>
-      </c>
-      <c r="W23" s="2">
-        <v>6.22497188600871</v>
-      </c>
-      <c r="X23" s="2">
-        <v>0.46443798485700399</v>
-      </c>
-      <c r="Y23" s="2">
-        <v>0.18432814038919701</v>
-      </c>
-      <c r="Z23" s="2">
-        <v>0.70490029069466198</v>
-      </c>
-      <c r="AA23" s="2">
-        <v>0.42196075107700698</v>
-      </c>
-      <c r="AB23" s="2">
-        <v>7.7067695459999502E-2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.75">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="B24" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="C24" t="s">
         <v>31</v>
@@ -3321,656 +3334,680 @@
         <v>0.11999999731779</v>
       </c>
       <c r="G24">
-        <v>463</v>
+        <v>492</v>
       </c>
       <c r="H24">
-        <v>438</v>
+        <v>493</v>
       </c>
       <c r="I24">
-        <v>379</v>
+        <v>470</v>
       </c>
       <c r="J24" s="2">
-        <v>55.559998758137198</v>
+        <v>59.039998680353101</v>
       </c>
       <c r="K24" s="2">
-        <v>52.559998825192402</v>
+        <v>59.159998677670899</v>
       </c>
       <c r="L24" s="2">
-        <v>45.479998983442698</v>
+        <v>56.399998739361699</v>
       </c>
       <c r="M24">
-        <v>379</v>
+        <v>470</v>
       </c>
       <c r="N24">
-        <v>340</v>
+        <v>409</v>
       </c>
       <c r="O24">
-        <v>338</v>
+        <v>408</v>
       </c>
       <c r="P24" s="2">
-        <v>0.115199994850158</v>
+        <v>0.100799995493888</v>
       </c>
       <c r="Q24" s="2">
-        <v>15.4655993086338</v>
+        <v>27.705598761463101</v>
       </c>
       <c r="R24" s="2">
-        <v>7.2921173210757599</v>
+        <v>13.406540231976701</v>
       </c>
       <c r="S24" s="2">
-        <v>2.9178599191496599</v>
+        <v>7.2227892634755397</v>
       </c>
       <c r="T24" s="2">
-        <v>4.1176173444915696</v>
+        <v>-3.6791164126064002</v>
       </c>
       <c r="U24" s="2">
-        <v>49.295073842977501</v>
+        <v>48.885386689612801</v>
       </c>
       <c r="V24" s="2">
-        <v>27.941382085633101</v>
+        <v>11.991644925359401</v>
       </c>
       <c r="W24" s="2">
-        <v>12.962633261614499</v>
+        <v>11.7091698601528</v>
       </c>
       <c r="X24" s="2">
-        <v>0.29751838004983699</v>
+        <v>0.65799297987812999</v>
       </c>
       <c r="Y24" s="2">
-        <v>0.200785499560584</v>
+        <v>0.245436926061702</v>
       </c>
       <c r="Z24" s="2">
-        <v>0.68401124997850304</v>
+        <v>0.62831853071795796</v>
       </c>
       <c r="AA24" s="2">
-        <v>0.45988044872012401</v>
+        <v>0.45913242350329603</v>
       </c>
       <c r="AB24" s="2">
-        <v>0.108664365284508</v>
+        <v>8.0821992081826305E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.75">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="B25" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C25" t="s">
+        <v>31</v>
+      </c>
+      <c r="D25" s="2">
+        <v>0.109999999403953</v>
+      </c>
+      <c r="E25" s="2">
+        <v>0.109999999403953</v>
+      </c>
+      <c r="F25" s="2">
+        <v>0.109999999403953</v>
+      </c>
+      <c r="G25">
+        <v>552</v>
+      </c>
+      <c r="H25">
+        <v>363</v>
+      </c>
+      <c r="I25">
+        <v>459</v>
+      </c>
+      <c r="J25" s="2">
+        <v>60.719999670982297</v>
+      </c>
+      <c r="K25" s="2">
+        <v>39.929999783635097</v>
+      </c>
+      <c r="L25" s="2">
+        <v>50.489999726414602</v>
+      </c>
+      <c r="M25">
+        <v>459</v>
+      </c>
+      <c r="N25">
+        <v>250</v>
+      </c>
+      <c r="O25">
+        <v>250</v>
+      </c>
+      <c r="P25" s="2">
+        <v>0.55659999396800997</v>
+      </c>
+      <c r="Q25" s="2">
+        <v>19.6261997873067</v>
+      </c>
+      <c r="R25" s="2">
+        <v>12.8599766606337</v>
+      </c>
+      <c r="S25" s="2">
+        <v>3.5533952235611399</v>
+      </c>
+      <c r="T25" s="2">
+        <v>0.62020326684607796</v>
+      </c>
+      <c r="U25" s="2">
+        <v>26.150628333948799</v>
+      </c>
+      <c r="V25" s="2">
+        <v>14.951127457630699</v>
+      </c>
+      <c r="W25" s="2">
+        <v>4.90757399859252</v>
+      </c>
+      <c r="X25" s="2">
+        <v>0.35364935625114202</v>
+      </c>
+      <c r="Y25" s="2">
+        <v>0.20877827064899801</v>
+      </c>
+      <c r="Z25" s="2">
+        <v>0.85510805955698499</v>
+      </c>
+      <c r="AA25" s="2">
+        <v>0.43121663980741198</v>
+      </c>
+      <c r="AB25" s="2">
+        <v>0.14659196018929799</v>
+      </c>
+    </row>
+    <row r="26" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>73</v>
+      </c>
+      <c r="B26" t="s">
+        <v>74</v>
+      </c>
+      <c r="C26" t="s">
         <v>34</v>
       </c>
-      <c r="D25" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="E25" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="F25" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="G25">
-        <v>533</v>
-      </c>
-      <c r="H25">
-        <v>464</v>
-      </c>
-      <c r="I25">
-        <v>440</v>
-      </c>
-      <c r="J25" s="2">
-        <v>63.959998570382503</v>
-      </c>
-      <c r="K25" s="2">
-        <v>55.679998755455003</v>
-      </c>
-      <c r="L25" s="2">
-        <v>52.799998819827998</v>
-      </c>
-      <c r="M25">
-        <v>440</v>
-      </c>
-      <c r="N25">
-        <v>364</v>
-      </c>
-      <c r="O25">
-        <v>337</v>
-      </c>
-      <c r="P25" s="2">
-        <v>1.7423999221086499</v>
-      </c>
-      <c r="Q25" s="2">
-        <v>50.500797742438301</v>
-      </c>
-      <c r="R25" s="2">
-        <v>32.348016136348498</v>
-      </c>
-      <c r="S25" s="2">
-        <v>8.1421562230672802</v>
-      </c>
-      <c r="T25" s="2">
-        <v>-20.527470393122201</v>
-      </c>
-      <c r="U25" s="2">
-        <v>6.2944695376730397</v>
-      </c>
-      <c r="V25" s="2">
-        <v>-8.72487054063307</v>
-      </c>
-      <c r="W25" s="2">
-        <v>7.6323523358807002</v>
-      </c>
-      <c r="X25" s="2">
-        <v>1.4129613132535499</v>
-      </c>
-      <c r="Y25" s="2">
-        <v>0.13514368714610001</v>
-      </c>
-      <c r="Z25" s="2">
-        <v>0.71858735554700304</v>
-      </c>
-      <c r="AA25" s="2">
-        <v>0.35762653325822802</v>
-      </c>
-      <c r="AB25" s="2">
-        <v>8.5734654338940702E-2</v>
+      <c r="D26" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E26" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F26" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G26">
+        <v>457</v>
+      </c>
+      <c r="H26">
+        <v>503</v>
+      </c>
+      <c r="I26">
+        <v>530</v>
+      </c>
+      <c r="J26" s="2">
+        <v>54.839998774230402</v>
+      </c>
+      <c r="K26" s="2">
+        <v>60.359998650848802</v>
+      </c>
+      <c r="L26" s="2">
+        <v>63.599998578429201</v>
+      </c>
+      <c r="M26">
+        <v>530</v>
+      </c>
+      <c r="N26">
+        <v>348</v>
+      </c>
+      <c r="O26">
+        <v>348</v>
+      </c>
+      <c r="P26" s="2">
+        <v>0.41759998133182502</v>
+      </c>
+      <c r="Q26" s="2">
+        <v>19.915199109721101</v>
+      </c>
+      <c r="R26" s="2">
+        <v>11.121599502825701</v>
+      </c>
+      <c r="S26" s="2">
+        <v>5.7592023770084904</v>
+      </c>
+      <c r="T26" s="2">
+        <v>-19.800098712087902</v>
+      </c>
+      <c r="U26" s="2">
+        <v>1.55906942884642</v>
+      </c>
+      <c r="V26" s="2">
+        <v>-6.89808119767501</v>
+      </c>
+      <c r="W26" s="2">
+        <v>6.22497188600871</v>
+      </c>
+      <c r="X26" s="2">
+        <v>0.46443798485700399</v>
+      </c>
+      <c r="Y26" s="2">
+        <v>0.18432814038919701</v>
+      </c>
+      <c r="Z26" s="2">
+        <v>0.70490029069466198</v>
+      </c>
+      <c r="AA26" s="2">
+        <v>0.42196075107700698</v>
+      </c>
+      <c r="AB26" s="2">
+        <v>7.7067695459999502E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.75">
-      <c r="A26" t="s">
-        <v>79</v>
-      </c>
-      <c r="B26" t="s">
-        <v>80</v>
-      </c>
-      <c r="C26" t="s">
+    <row r="27" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>39</v>
+      </c>
+      <c r="B27" t="s">
+        <v>40</v>
+      </c>
+      <c r="C27" t="s">
         <v>31</v>
       </c>
-      <c r="D26" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="E26" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="F26" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="G26">
-        <v>507</v>
-      </c>
-      <c r="H26">
-        <v>480</v>
-      </c>
-      <c r="I26">
-        <v>567</v>
-      </c>
-      <c r="J26" s="2">
-        <v>60.839998640120001</v>
-      </c>
-      <c r="K26" s="2">
-        <v>57.599998712539602</v>
-      </c>
-      <c r="L26" s="2">
-        <v>68.039998479187403</v>
-      </c>
-      <c r="M26">
-        <v>567</v>
-      </c>
-      <c r="N26">
-        <v>473</v>
-      </c>
-      <c r="O26">
-        <v>473</v>
-      </c>
-      <c r="P26" s="2">
-        <v>0.115199994850158</v>
-      </c>
-      <c r="Q26" s="2">
-        <v>72.590396754956203</v>
-      </c>
-      <c r="R26" s="2">
-        <v>32.385294112518103</v>
-      </c>
-      <c r="S26" s="2">
-        <v>15.326562163500499</v>
-      </c>
-      <c r="T26" s="2">
-        <v>-1.59280688897673</v>
-      </c>
-      <c r="U26" s="2">
-        <v>38.702431399926198</v>
-      </c>
-      <c r="V26" s="2">
-        <v>12.2910171632528</v>
-      </c>
-      <c r="W26" s="2">
-        <v>11.8919504088847</v>
-      </c>
-      <c r="X26" s="2">
-        <v>1.8381892527398001</v>
-      </c>
-      <c r="Y26" s="2">
-        <v>0.11394954450048</v>
-      </c>
-      <c r="Z26" s="2">
-        <v>0.54872876285580996</v>
-      </c>
-      <c r="AA26" s="2">
-        <v>0.426328774527649</v>
-      </c>
-      <c r="AB26" s="2">
-        <v>6.4062039505979093E-2</v>
+      <c r="D27" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E27" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F27" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G27">
+        <v>493</v>
+      </c>
+      <c r="H27">
+        <v>444</v>
+      </c>
+      <c r="I27">
+        <v>415</v>
+      </c>
+      <c r="J27" s="2">
+        <v>59.159998677670899</v>
+      </c>
+      <c r="K27" s="2">
+        <v>53.279998809099197</v>
+      </c>
+      <c r="L27" s="2">
+        <v>49.799998886883202</v>
+      </c>
+      <c r="M27">
+        <v>415</v>
+      </c>
+      <c r="N27">
+        <v>276</v>
+      </c>
+      <c r="O27">
+        <v>276</v>
+      </c>
+      <c r="P27" s="2">
+        <v>0.84959996201992005</v>
+      </c>
+      <c r="Q27" s="2">
+        <v>17.279999227523799</v>
+      </c>
+      <c r="R27" s="2">
+        <v>10.401077795905101</v>
+      </c>
+      <c r="S27" s="2">
+        <v>2.71633372610582</v>
+      </c>
+      <c r="T27" s="2">
+        <v>22.781328024984099</v>
+      </c>
+      <c r="U27" s="2">
+        <v>47.723491609628702</v>
+      </c>
+      <c r="V27" s="2">
+        <v>40.149546052521799</v>
+      </c>
+      <c r="W27" s="2">
+        <v>7.5920641408914999</v>
+      </c>
+      <c r="X27" s="2">
+        <v>0.34448368890056702</v>
+      </c>
+      <c r="Y27" s="2">
+        <v>0.38660823879890699</v>
+      </c>
+      <c r="Z27" s="2">
+        <v>0.65624379874986705</v>
+      </c>
+      <c r="AA27" s="2">
+        <v>0.50671206800679403</v>
+      </c>
+      <c r="AB27" s="2">
+        <v>5.0269621417554498E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.75">
-      <c r="A27" t="s">
-        <v>81</v>
-      </c>
-      <c r="B27" t="s">
-        <v>82</v>
-      </c>
-      <c r="C27" t="s">
+    <row r="28" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>37</v>
+      </c>
+      <c r="B28" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" t="s">
         <v>34</v>
       </c>
-      <c r="D27" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="E27" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="F27" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="G27">
-        <v>488</v>
-      </c>
-      <c r="H27">
-        <v>503</v>
-      </c>
-      <c r="I27">
-        <v>544</v>
-      </c>
-      <c r="J27" s="2">
-        <v>58.559998691082001</v>
-      </c>
-      <c r="K27" s="2">
-        <v>60.359998650848802</v>
-      </c>
-      <c r="L27" s="2">
-        <v>65.279998540878296</v>
-      </c>
-      <c r="M27">
-        <v>544</v>
-      </c>
-      <c r="N27">
-        <v>413</v>
-      </c>
-      <c r="O27">
-        <v>413</v>
-      </c>
-      <c r="P27" s="2">
-        <v>4.3199998068809503E-2</v>
-      </c>
-      <c r="Q27" s="2">
-        <v>33.883198485302898</v>
-      </c>
-      <c r="R27" s="2">
-        <v>16.1630404396833</v>
-      </c>
-      <c r="S27" s="2">
-        <v>5.5449052384811104</v>
-      </c>
-      <c r="T27" s="2">
-        <v>-30.113181857117699</v>
-      </c>
-      <c r="U27" s="2">
-        <v>14.5372308886172</v>
-      </c>
-      <c r="V27" s="2">
-        <v>-2.2214572979969098</v>
-      </c>
-      <c r="W27" s="2">
-        <v>10.317174022222501</v>
-      </c>
-      <c r="X27" s="2">
-        <v>0.80104026628606195</v>
-      </c>
-      <c r="Y27" s="2">
-        <v>0.21681631811889299</v>
-      </c>
-      <c r="Z27" s="2">
-        <v>0.73100770886853905</v>
-      </c>
-      <c r="AA27" s="2">
-        <v>0.40499463756417198</v>
-      </c>
-      <c r="AB27" s="2">
-        <v>0.12384299345529901</v>
+      <c r="D28" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E28" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F28" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G28">
+        <v>501</v>
+      </c>
+      <c r="H28">
+        <v>516</v>
+      </c>
+      <c r="I28">
+        <v>625</v>
+      </c>
+      <c r="J28" s="2">
+        <v>60.119998656213198</v>
+      </c>
+      <c r="K28" s="2">
+        <v>61.919998615980099</v>
+      </c>
+      <c r="L28" s="2">
+        <v>74.999998323619295</v>
+      </c>
+      <c r="M28">
+        <v>625</v>
+      </c>
+      <c r="N28">
+        <v>189</v>
+      </c>
+      <c r="O28">
+        <v>189</v>
+      </c>
+      <c r="P28" s="2">
+        <v>0.14399999356269799</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>19.1663991431951</v>
+      </c>
+      <c r="R28" s="2">
+        <v>10.301713825191699</v>
+      </c>
+      <c r="S28" s="2">
+        <v>5.88375254411425</v>
+      </c>
+      <c r="T28" s="2">
+        <v>5.6429962496727804</v>
+      </c>
+      <c r="U28" s="2">
+        <v>9.4515843436410396</v>
+      </c>
+      <c r="V28" s="2">
+        <v>7.4012167862119904</v>
+      </c>
+      <c r="W28" s="2">
+        <v>0.92234835893643996</v>
+      </c>
+      <c r="X28" s="2">
+        <v>0.233642864333024</v>
+      </c>
+      <c r="Y28" s="2">
+        <v>0.17990560012635001</v>
+      </c>
+      <c r="Z28" s="2">
+        <v>0.75630934253087601</v>
+      </c>
+      <c r="AA28" s="2">
+        <v>0.48534067754822702</v>
+      </c>
+      <c r="AB28" s="2">
+        <v>9.7658132006584297E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:28" x14ac:dyDescent="0.75">
-      <c r="A28" t="s">
-        <v>83</v>
-      </c>
-      <c r="B28" t="s">
-        <v>84</v>
-      </c>
-      <c r="C28" t="s">
-        <v>31</v>
-      </c>
-      <c r="D28" s="2">
-        <v>0.109999999403953</v>
-      </c>
-      <c r="E28" s="2">
-        <v>0.109999999403953</v>
-      </c>
-      <c r="F28" s="2">
-        <v>0.109999999403953</v>
-      </c>
-      <c r="G28">
-        <v>552</v>
-      </c>
-      <c r="H28">
-        <v>363</v>
-      </c>
-      <c r="I28">
-        <v>459</v>
-      </c>
-      <c r="J28" s="2">
-        <v>60.719999670982297</v>
-      </c>
-      <c r="K28" s="2">
-        <v>39.929999783635097</v>
-      </c>
-      <c r="L28" s="2">
-        <v>50.489999726414602</v>
-      </c>
-      <c r="M28">
-        <v>459</v>
-      </c>
-      <c r="N28">
-        <v>250</v>
-      </c>
-      <c r="O28">
-        <v>250</v>
-      </c>
-      <c r="P28" s="2">
-        <v>0.55659999396800997</v>
-      </c>
-      <c r="Q28" s="2">
-        <v>19.6261997873067</v>
-      </c>
-      <c r="R28" s="2">
-        <v>12.8599766606337</v>
-      </c>
-      <c r="S28" s="2">
-        <v>3.5533952235611399</v>
-      </c>
-      <c r="T28" s="2">
-        <v>0.62020326684607796</v>
-      </c>
-      <c r="U28" s="2">
-        <v>26.150628333948799</v>
-      </c>
-      <c r="V28" s="2">
-        <v>14.951127457630699</v>
-      </c>
-      <c r="W28" s="2">
-        <v>4.90757399859252</v>
-      </c>
-      <c r="X28" s="2">
-        <v>0.35364935625114202</v>
-      </c>
-      <c r="Y28" s="2">
-        <v>0.20877827064899801</v>
-      </c>
-      <c r="Z28" s="2">
-        <v>0.85510805955698499</v>
-      </c>
-      <c r="AA28" s="2">
-        <v>0.43121663980741198</v>
-      </c>
-      <c r="AB28" s="2">
-        <v>0.14659196018929799</v>
-      </c>
-    </row>
-    <row r="29" spans="1:28" x14ac:dyDescent="0.75">
+    <row r="29" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="B29" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="C29" t="s">
         <v>34</v>
       </c>
       <c r="D29" s="2">
-        <v>0.109999999403953</v>
+        <v>0.11999999731779</v>
       </c>
       <c r="E29" s="2">
-        <v>0.109999999403953</v>
+        <v>0.11999999731779</v>
       </c>
       <c r="F29" s="2">
-        <v>0.109999999403953</v>
+        <v>0.11999999731779</v>
       </c>
       <c r="G29">
-        <v>604</v>
+        <v>509</v>
       </c>
       <c r="H29">
-        <v>482</v>
+        <v>419</v>
       </c>
       <c r="I29">
-        <v>546</v>
+        <v>470</v>
       </c>
       <c r="J29" s="2">
-        <v>66.439999639987903</v>
+        <v>61.079998634755597</v>
       </c>
       <c r="K29" s="2">
-        <v>53.019999712705598</v>
+        <v>50.279998876154401</v>
       </c>
       <c r="L29" s="2">
-        <v>60.059999674558597</v>
+        <v>56.399998739361699</v>
       </c>
       <c r="M29">
-        <v>546</v>
+        <v>470</v>
       </c>
       <c r="N29">
-        <v>376</v>
+        <v>421</v>
       </c>
       <c r="O29">
-        <v>376</v>
+        <v>421</v>
       </c>
       <c r="P29" s="2">
-        <v>0.108899998819828</v>
+        <v>0.17279999227523801</v>
       </c>
       <c r="Q29" s="2">
-        <v>41.865999546289402</v>
+        <v>19.238399139976501</v>
       </c>
       <c r="R29" s="2">
-        <v>18.786537030448901</v>
+        <v>9.4470494589191194</v>
       </c>
       <c r="S29" s="2">
-        <v>9.9718519030673392</v>
+        <v>4.4674063575587502</v>
       </c>
       <c r="T29" s="2">
-        <v>-18.664611344916999</v>
+        <v>-37.377476810110601</v>
       </c>
       <c r="U29" s="2">
-        <v>8.4478220753991895</v>
+        <v>8.8260465440543907</v>
       </c>
       <c r="V29" s="2">
-        <v>-8.6137667186061506</v>
+        <v>-9.3330666501601804</v>
       </c>
       <c r="W29" s="2">
-        <v>8.9614095681574799</v>
+        <v>14.532382732052</v>
       </c>
       <c r="X29" s="2">
-        <v>0.77701116736905196</v>
+        <v>0.47726492799689102</v>
       </c>
       <c r="Y29" s="2">
-        <v>0.28972257847031402</v>
+        <v>0.17896940301683301</v>
       </c>
       <c r="Z29" s="2">
-        <v>1</v>
+        <v>0.95660952773668395</v>
       </c>
       <c r="AA29" s="2">
-        <v>0.53287827651128705</v>
+        <v>0.37852913096401303</v>
       </c>
       <c r="AB29" s="2">
-        <v>8.59954147501025E-2</v>
+        <v>9.7776851486295405E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:28" x14ac:dyDescent="0.75">
+    <row r="30" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>87</v>
+        <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="C30" t="s">
+        <v>34</v>
+      </c>
+      <c r="D30" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E30" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F30" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G30">
+        <v>496</v>
+      </c>
+      <c r="H30">
+        <v>404</v>
+      </c>
+      <c r="I30">
+        <v>396</v>
+      </c>
+      <c r="J30" s="2">
+        <v>59.5199986696243</v>
+      </c>
+      <c r="K30" s="2">
+        <v>48.479998916387501</v>
+      </c>
+      <c r="L30" s="2">
+        <v>47.519998937845202</v>
+      </c>
+      <c r="M30">
+        <v>396</v>
+      </c>
+      <c r="N30">
+        <v>257</v>
+      </c>
+      <c r="O30">
+        <v>257</v>
+      </c>
+      <c r="P30" s="2">
+        <v>0.34559998455047602</v>
+      </c>
+      <c r="Q30" s="2">
+        <v>16.3151992706537</v>
+      </c>
+      <c r="R30" s="2">
+        <v>8.9000400690632606</v>
+      </c>
+      <c r="S30" s="2">
+        <v>3.2383094064033</v>
+      </c>
+      <c r="T30" s="2">
+        <v>-17.718737569616302</v>
+      </c>
+      <c r="U30" s="2">
+        <v>1.1242703657935</v>
+      </c>
+      <c r="V30" s="2">
+        <v>-5.1390677634215702</v>
+      </c>
+      <c r="W30" s="2">
+        <v>5.4008666819821496</v>
+      </c>
+      <c r="X30" s="2">
+        <v>0.27447722959486598</v>
+      </c>
+      <c r="Y30" s="2">
+        <v>0.28683732101911702</v>
+      </c>
+      <c r="Z30" s="2">
+        <v>0.75398223686154997</v>
+      </c>
+      <c r="AA30" s="2">
+        <v>0.45436411435693602</v>
+      </c>
+      <c r="AB30" s="2">
+        <v>9.5494725170903294E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>75</v>
+      </c>
+      <c r="B31" t="s">
+        <v>76</v>
+      </c>
+      <c r="C31" t="s">
         <v>31</v>
       </c>
-      <c r="D30" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="E30" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="F30" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="G30">
-        <v>559</v>
-      </c>
-      <c r="H30">
-        <v>444</v>
-      </c>
-      <c r="I30">
-        <v>611</v>
-      </c>
-      <c r="J30" s="2">
-        <v>67.079998500645104</v>
-      </c>
-      <c r="K30" s="2">
-        <v>53.279998809099197</v>
-      </c>
-      <c r="L30" s="2">
-        <v>73.319998361170207</v>
-      </c>
-      <c r="M30">
-        <v>611</v>
-      </c>
-      <c r="N30">
-        <v>0</v>
-      </c>
-      <c r="O30">
-        <v>0</v>
-      </c>
-      <c r="P30" s="2"/>
-      <c r="Q30" s="2"/>
-      <c r="R30" s="2"/>
-      <c r="S30" s="2"/>
-      <c r="T30" s="2"/>
-      <c r="U30" s="2"/>
-      <c r="V30" s="2"/>
-      <c r="W30" s="2"/>
-      <c r="X30" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y30" s="2"/>
-      <c r="Z30" s="2"/>
-      <c r="AA30" s="2"/>
-      <c r="AB30" s="2"/>
+      <c r="D31" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="E31" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="F31" s="2">
+        <v>0.11999999731779</v>
+      </c>
+      <c r="G31">
+        <v>463</v>
+      </c>
+      <c r="H31">
+        <v>438</v>
+      </c>
+      <c r="I31">
+        <v>379</v>
+      </c>
+      <c r="J31" s="2">
+        <v>55.559998758137198</v>
+      </c>
+      <c r="K31" s="2">
+        <v>52.559998825192402</v>
+      </c>
+      <c r="L31" s="2">
+        <v>45.479998983442698</v>
+      </c>
+      <c r="M31">
+        <v>379</v>
+      </c>
+      <c r="N31">
+        <v>340</v>
+      </c>
+      <c r="O31">
+        <v>338</v>
+      </c>
+      <c r="P31" s="2">
+        <v>0.115199994850158</v>
+      </c>
+      <c r="Q31" s="2">
+        <v>15.4655993086338</v>
+      </c>
+      <c r="R31" s="2">
+        <v>7.2921173210757599</v>
+      </c>
+      <c r="S31" s="2">
+        <v>2.9178599191496599</v>
+      </c>
+      <c r="T31" s="2">
+        <v>4.1176173444915696</v>
+      </c>
+      <c r="U31" s="2">
+        <v>49.295073842977501</v>
+      </c>
+      <c r="V31" s="2">
+        <v>27.941382085633101</v>
+      </c>
+      <c r="W31" s="2">
+        <v>12.962633261614499</v>
+      </c>
+      <c r="X31" s="2">
+        <v>0.29751838004983699</v>
+      </c>
+      <c r="Y31" s="2">
+        <v>0.200785499560584</v>
+      </c>
+      <c r="Z31" s="2">
+        <v>0.68401124997850304</v>
+      </c>
+      <c r="AA31" s="2">
+        <v>0.45988044872012401</v>
+      </c>
+      <c r="AB31" s="2">
+        <v>0.108664365284508</v>
+      </c>
     </row>
-    <row r="31" spans="1:28" x14ac:dyDescent="0.75">
-      <c r="A31" t="s">
-        <v>89</v>
-      </c>
-      <c r="B31" t="s">
-        <v>90</v>
-      </c>
-      <c r="C31" t="s">
-        <v>34</v>
-      </c>
-      <c r="D31" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="E31" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="F31" s="2">
-        <v>0.11999999731779</v>
-      </c>
-      <c r="G31">
-        <v>588</v>
-      </c>
-      <c r="H31">
-        <v>514</v>
-      </c>
-      <c r="I31">
-        <v>696</v>
-      </c>
-      <c r="J31" s="2">
-        <v>70.559998422861099</v>
-      </c>
-      <c r="K31" s="2">
-        <v>61.679998621344502</v>
-      </c>
-      <c r="L31" s="2">
-        <v>83.519998133182497</v>
-      </c>
-      <c r="M31">
-        <v>696</v>
-      </c>
-      <c r="N31">
-        <v>530</v>
-      </c>
-      <c r="O31">
-        <v>530</v>
-      </c>
-      <c r="P31" s="2">
-        <v>0.54719997553825395</v>
-      </c>
-      <c r="Q31" s="2">
-        <v>40.535998187899601</v>
-      </c>
-      <c r="R31" s="2">
-        <v>28.883790406907099</v>
-      </c>
-      <c r="S31" s="2">
-        <v>7.8649864410657599</v>
-      </c>
-      <c r="T31" s="2">
-        <v>-24.743954745608399</v>
-      </c>
-      <c r="U31" s="2">
-        <v>9.7046363882575104</v>
-      </c>
-      <c r="V31" s="2">
-        <v>0.83436034278634796</v>
-      </c>
-      <c r="W31" s="2">
-        <v>8.0313582978660207</v>
-      </c>
-      <c r="X31" s="2">
-        <v>1.83700902881894</v>
-      </c>
-      <c r="Y31" s="2">
-        <v>0.11867453863633599</v>
-      </c>
-      <c r="Z31" s="2">
-        <v>0.70639361441663895</v>
-      </c>
-      <c r="AA31" s="2">
-        <v>0.39402604452571399</v>
-      </c>
-      <c r="AB31" s="2">
-        <v>0.145607079988959</v>
-      </c>
-    </row>
-    <row r="32" spans="1:28" x14ac:dyDescent="0.75">
+    <row r="32" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="B32" t="s">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="C32" t="s">
         <v>31</v>
@@ -3985,81 +4022,81 @@
         <v>0.11999999731779</v>
       </c>
       <c r="G32">
-        <v>536</v>
+        <v>500</v>
       </c>
       <c r="H32">
-        <v>521</v>
+        <v>442</v>
       </c>
       <c r="I32">
-        <v>584</v>
+        <v>479</v>
       </c>
       <c r="J32" s="2">
-        <v>64.319998562335897</v>
+        <v>59.9999986588954</v>
       </c>
       <c r="K32" s="2">
-        <v>62.519998602569103</v>
+        <v>53.039998814463601</v>
       </c>
       <c r="L32" s="2">
-        <v>70.079998433589907</v>
+        <v>57.479998715221797</v>
       </c>
       <c r="M32">
-        <v>584</v>
+        <v>479</v>
       </c>
       <c r="N32">
-        <v>393</v>
+        <v>281</v>
       </c>
       <c r="O32">
-        <v>381</v>
+        <v>281</v>
       </c>
       <c r="P32" s="2">
-        <v>0.115199994850158</v>
+        <v>0.100799995493888</v>
       </c>
       <c r="Q32" s="2">
-        <v>60.868797278952599</v>
+        <v>10.0655995500326</v>
       </c>
       <c r="R32" s="2">
-        <v>46.3905322773265</v>
+        <v>6.2332523903910397</v>
       </c>
       <c r="S32" s="2">
-        <v>13.435491339866999</v>
+        <v>1.6164454200715701</v>
       </c>
       <c r="T32" s="2">
-        <v>-3.1914997723557601</v>
+        <v>5.5762378785484499</v>
       </c>
       <c r="U32" s="2">
-        <v>45.938782762473998</v>
+        <v>52.288517561874002</v>
       </c>
       <c r="V32" s="2">
-        <v>19.107941579070602</v>
+        <v>28.889137936259299</v>
       </c>
       <c r="W32" s="2">
-        <v>12.049508977116099</v>
+        <v>15.527761680313899</v>
       </c>
       <c r="X32" s="2">
-        <v>2.18777745329808</v>
+        <v>0.210185265905978</v>
       </c>
       <c r="Y32" s="2">
-        <v>0.23619153925271799</v>
+        <v>0.50060688730810599</v>
       </c>
       <c r="Z32" s="2">
-        <v>0.69380443818948101</v>
+        <v>0.87266462599716399</v>
       </c>
       <c r="AA32" s="2">
-        <v>0.56888181700722096</v>
+        <v>0.63383746204019498</v>
       </c>
       <c r="AB32" s="2">
-        <v>7.5158251711053697E-2</v>
+        <v>5.19615440898075E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:28" x14ac:dyDescent="0.75">
+    <row r="33" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B33" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C33" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D33" s="2">
         <v>0.11999999731779</v>
@@ -4071,101 +4108,82 @@
         <v>0.11999999731779</v>
       </c>
       <c r="G33">
-        <v>512</v>
+        <v>559</v>
       </c>
       <c r="H33">
-        <v>430</v>
+        <v>444</v>
       </c>
       <c r="I33">
-        <v>452</v>
+        <v>611</v>
       </c>
       <c r="J33" s="2">
-        <v>61.439998626708899</v>
+        <v>67.079998500645104</v>
       </c>
       <c r="K33" s="2">
-        <v>51.599998846650102</v>
+        <v>53.279998809099197</v>
       </c>
       <c r="L33" s="2">
-        <v>54.239998787641497</v>
+        <v>73.319998361170207</v>
       </c>
       <c r="M33">
-        <v>452</v>
+        <v>611</v>
       </c>
       <c r="N33">
-        <v>398</v>
+        <v>0</v>
       </c>
       <c r="O33">
-        <v>398</v>
-      </c>
-      <c r="P33" s="2">
-        <v>4.3199998068809503E-2</v>
-      </c>
-      <c r="Q33" s="2">
-        <v>83.807996253490401</v>
-      </c>
-      <c r="R33" s="2">
-        <v>67.971072338340505</v>
-      </c>
-      <c r="S33" s="2">
-        <v>11.2770149298498</v>
-      </c>
-      <c r="T33" s="2">
-        <v>-27.615261894174001</v>
-      </c>
-      <c r="U33" s="2">
-        <v>25.1242028815597</v>
-      </c>
-      <c r="V33" s="2">
-        <v>-15.5767199462778</v>
-      </c>
-      <c r="W33" s="2">
-        <v>7.5223077608496096</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="P33" s="2"/>
+      <c r="Q33" s="2"/>
+      <c r="R33" s="2"/>
+      <c r="S33" s="2"/>
+      <c r="T33" s="2"/>
+      <c r="U33" s="2"/>
+      <c r="V33" s="2"/>
+      <c r="W33" s="2"/>
       <c r="X33" s="2">
-        <v>3.2462983423187199</v>
-      </c>
-      <c r="Y33" s="2">
-        <v>9.7071870521207596E-2</v>
-      </c>
-      <c r="Z33" s="2">
-        <v>0.67490278273135096</v>
-      </c>
-      <c r="AA33" s="2">
-        <v>0.59877287891169595</v>
-      </c>
-      <c r="AB33" s="2">
-        <v>7.9645327854629494E-2</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y33" s="2"/>
+      <c r="Z33" s="2"/>
+      <c r="AA33" s="2"/>
+      <c r="AB33" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC33" xr:uid="{2DF80251-01B8-4EEE-BE3E-F00FCAF28141}"/>
+  <autoFilter ref="A1:AC33" xr:uid="{2DF80251-01B8-4EEE-BE3E-F00FCAF28141}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AC33">
+      <sortCondition descending="1" ref="R1:R33"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64BC1F98-15C7-469E-BB0C-F6C580CA5A51}">
   <dimension ref="A1:AC17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.27734375" customWidth="1"/>
-    <col min="2" max="2" width="23.27734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.28515625" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="5.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="12" width="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.27734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.0546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="23" max="28" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="3" customFormat="1" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:29" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -4254,7 +4272,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>95</v>
       </c>
@@ -4340,7 +4358,7 @@
         <v>2.1709773126873399E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>97</v>
       </c>
@@ -4426,7 +4444,7 @@
         <v>2.9033387234841199E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>99</v>
       </c>
@@ -4512,7 +4530,7 @@
         <v>3.0737380706046001E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>101</v>
       </c>
@@ -4598,7 +4616,7 @@
         <v>2.94832860439279E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>103</v>
       </c>
@@ -4684,7 +4702,7 @@
         <v>2.8671400953959598E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>105</v>
       </c>
@@ -4770,7 +4788,7 @@
         <v>3.5312200977370201E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>107</v>
       </c>
@@ -4856,7 +4874,7 @@
         <v>3.4875554338025E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>109</v>
       </c>
@@ -4942,7 +4960,7 @@
         <v>1.04365774813773E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>111</v>
       </c>
@@ -5028,7 +5046,7 @@
         <v>1.28319954015985E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>113</v>
       </c>
@@ -5114,7 +5132,7 @@
         <v>1.12107980906852E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>115</v>
       </c>
@@ -5200,7 +5218,7 @@
         <v>2.3938202604705999E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>117</v>
       </c>
@@ -5286,7 +5304,7 @@
         <v>2.1534144235893699E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>119</v>
       </c>
@@ -5372,7 +5390,7 @@
         <v>2.38454273633316E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>121</v>
       </c>
@@ -5458,7 +5476,7 @@
         <v>3.0213825574389001E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>123</v>
       </c>
@@ -5544,7 +5562,7 @@
         <v>2.9960233782089198E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.75">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>125</v>
       </c>

</xml_diff>